<commit_message>
feat(proje-kontrol): Faz 1 Adım 5 kodu ve yerel test ortamı (Karar 52-59; test yok, deploy yok)
- DB taslağı f1_adim5_ekran_rpc.sql: get_project_gantt alanları, save_area_wbs_links,
  set_tasks_classification, save_project_tasks (Ç-B), ağırlıksız kategori trigger'ları, Ç-6 RLS
- Karar 44: iptal etme de yalnızca admin/PM (AID A8b); f1_dogrulama R15 güncellendi, §7 R28-R31
- Yerel ortam: scripts/local-db (setup/seed), supabase/local; Playwright varsayılan hedef yerel
- İş Planı: Activity ID/disiplin/alan/WBS, toplu atama, Kod ata, sınıflandırma, iptal/yeniden aç
- Proje Ayarları › WBS ve Alanlar bileşenleri (ProjeDetay bağlantısı kullanıcı dosyası, Ek A)
- Sihirbaz: proje kodu, save_project_tasks önizlemesi, group_label korunur; Excel şablonu v8 (E13)
- Edge function kodu güncellendi, deploy edilmedi; canlıya hiçbir şey uygulanmadı

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/excel/fons-solar-proje-sablonu.xlsx
+++ b/public/excel/fons-solar-proje-sablonu.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="160">
   <si>
     <t xml:space="preserve">  FONS SOLAR   |   PROJE BİLGİLERİ</t>
   </si>
@@ -74,6 +74,12 @@
   </si>
   <si>
     <t>← Başlangıç ve bitiş tarihlerinden otomatik</t>
+  </si>
+  <si>
+    <t>Proje Kodu *</t>
+  </si>
+  <si>
+    <t>2-5 karakter, harfle başlar, büyük harf/rakam (ör. DYB). Sonradan değiştirilemez</t>
   </si>
   <si>
     <t>GÜÇ BİLGİLERİ</t>
@@ -428,7 +434,7 @@
     <t xml:space="preserve">  FONS SOLAR   |   KULLANIM KILAVUZU</t>
   </si>
   <si>
-    <t>Şablon v7 (03.08.2026: İş Kalemleri'nden Dashboard Göster/Sıra ve Kritik mi? kolonları kaldırıldı)</t>
+    <t>Şablon v8 (12.10.2026: Proje Bilgileri E13 Proje Kodu eklendi; ağırlıksız kategoriye görev yazılamaz)</t>
   </si>
   <si>
     <t>1️⃣</t>
@@ -438,6 +444,9 @@
   </si>
   <si>
     <t>Proje ID: küçük harf, boşluksuz, tire. Tür ve Durum dropdown. Toplam Gün otomatik.</t>
+  </si>
+  <si>
+    <t>Proje ID: küçük harf, boşluksuz, tire. Proje Kodu (E13): 2-5 karakter, harfle başlar, büyük harf/rakam (ör. DYB); yeni projede zorunlu, sonradan değiştirilemez. Mevcut projeyi güncellerken E13 projenin koduyla aynı olmalı, yoksa yükleme reddedilir. Tür ve Durum dropdown. Toplam Gün otomatik.</t>
   </si>
   <si>
     <t>2️⃣</t>
@@ -456,6 +465,9 @@
   </si>
   <si>
     <t>Genel proje ilerlemesi bu 10 sabit kategorinin ağırlıklı ortalamasıdır. Buradan veri içeri aktarılmaz — görevleri doğru Kategori'ye atamak yeterlidir.</t>
+  </si>
+  <si>
+    <t>Genel proje ilerlemesi ağırlık tablosundaki kategorilerin ağırlıklı ortalamasıdır. Buradan veri içeri aktarılmaz. Ağırlık tablosunda olmayan kategoriye görev yazılamaz: önce ağırlık tanımlayın, fiziksel değilse %0 girin.</t>
   </si>
   <si>
     <t>4️⃣</t>
@@ -1277,9 +1289,21 @@
         <v>17</v>
       </c>
     </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13" s="5"/>
+      <c r="F13"/>
+      <c r="H13" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B14"/>
       <c r="C14"/>
@@ -1295,43 +1319,43 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C15"/>
       <c r="D15"/>
       <c r="E15" s="5"/>
       <c r="F15" s="6"/>
       <c r="H15" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16" s="5"/>
       <c r="F16" s="6"/>
       <c r="H16" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C17"/>
       <c r="D17"/>
       <c r="E17" s="5"/>
       <c r="F17" s="6"/>
       <c r="H17" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1347,52 +1371,52 @@
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C20"/>
       <c r="D20"/>
       <c r="E20" s="5"/>
       <c r="F20" s="6"/>
       <c r="H20" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J20" s="5"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C21"/>
       <c r="D21"/>
       <c r="E21" s="5"/>
       <c r="F21" s="6"/>
       <c r="H21" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J21" s="5"/>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C22"/>
       <c r="D22"/>
       <c r="E22" s="5"/>
       <c r="F22" s="6"/>
       <c r="H22" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="J22" s="5"/>
     </row>
     <row r="23" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H23" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J23" s="5"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B25"/>
       <c r="C25"/>
@@ -1407,7 +1431,7 @@
       <c r="L25"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="36">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A4:L4"/>
@@ -1427,6 +1451,8 @@
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:F13"/>
     <mergeCell ref="A14:L14"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="E15:F15"/>
@@ -1443,7 +1469,10 @@
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="A25:L25"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Proje kodu" error="2-5 karakter, harfle başlar, yalnızca büyük harf ve rakam (ör. DYB, ADN1)." sqref="E13">
+      <formula1>AND(LEN(E13)&gt;=2,LEN(E13)&lt;=5,EXACT(E13,UPPER(E13)),ISERROR(VALUE(LEFT(E13,1))))</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E8">
       <formula1>"Arazi GES,Endüstriyel Çatı GES,Evsel GES"</formula1>
     </dataValidation>
@@ -1514,54 +1543,54 @@
       <c r="Q2"/>
       <c r="R2"/>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>11</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -1581,7 +1610,7 @@
       <c r="N5" s="10"/>
       <c r="O5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -1601,7 +1630,7 @@
       <c r="N6" s="10"/>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -1621,7 +1650,7 @@
       <c r="N7" s="10"/>
       <c r="O7" s="10"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -1641,7 +1670,7 @@
       <c r="N8" s="10"/>
       <c r="O8" s="10"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -1661,7 +1690,7 @@
       <c r="N9" s="10"/>
       <c r="O9" s="10"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -1681,7 +1710,7 @@
       <c r="N10" s="10"/>
       <c r="O10" s="10"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -1701,7 +1730,7 @@
       <c r="N11" s="10"/>
       <c r="O11" s="10"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -1721,7 +1750,7 @@
       <c r="N12" s="10"/>
       <c r="O12" s="10"/>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1741,7 +1770,7 @@
       <c r="N13" s="10"/>
       <c r="O13" s="10"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -1761,7 +1790,7 @@
       <c r="N14" s="10"/>
       <c r="O14" s="10"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -1781,7 +1810,7 @@
       <c r="N15" s="10"/>
       <c r="O15" s="10"/>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -1801,7 +1830,7 @@
       <c r="N16" s="10"/>
       <c r="O16" s="10"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -1821,7 +1850,7 @@
       <c r="N17" s="10"/>
       <c r="O17" s="10"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -1841,7 +1870,7 @@
       <c r="N18" s="10"/>
       <c r="O18" s="10"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="10"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -1861,7 +1890,7 @@
       <c r="N19" s="10"/>
       <c r="O19" s="10"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -1881,7 +1910,7 @@
       <c r="N20" s="10"/>
       <c r="O20" s="10"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -1901,7 +1930,7 @@
       <c r="N21" s="10"/>
       <c r="O21" s="10"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -1921,7 +1950,7 @@
       <c r="N22" s="10"/>
       <c r="O22" s="10"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
@@ -1941,7 +1970,7 @@
       <c r="N23" s="10"/>
       <c r="O23" s="10"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -1961,7 +1990,7 @@
       <c r="N24" s="10"/>
       <c r="O24" s="10"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -1981,7 +2010,7 @@
       <c r="N25" s="10"/>
       <c r="O25" s="10"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -2001,7 +2030,7 @@
       <c r="N26" s="10"/>
       <c r="O26" s="10"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -2021,7 +2050,7 @@
       <c r="N27" s="10"/>
       <c r="O27" s="10"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -2041,7 +2070,7 @@
       <c r="N28" s="10"/>
       <c r="O28" s="10"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -2061,7 +2090,7 @@
       <c r="N29" s="10"/>
       <c r="O29" s="10"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -2081,7 +2110,7 @@
       <c r="N30" s="10"/>
       <c r="O30" s="10"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
@@ -2101,7 +2130,7 @@
       <c r="N31" s="10"/>
       <c r="O31" s="10"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
@@ -2121,7 +2150,7 @@
       <c r="N32" s="10"/>
       <c r="O32" s="10"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
@@ -2141,7 +2170,7 @@
       <c r="N33" s="10"/>
       <c r="O33" s="10"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -2161,7 +2190,7 @@
       <c r="N34" s="10"/>
       <c r="O34" s="10"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -2181,7 +2210,7 @@
       <c r="N35" s="10"/>
       <c r="O35" s="10"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
@@ -2201,7 +2230,7 @@
       <c r="N36" s="10"/>
       <c r="O36" s="10"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -2221,7 +2250,7 @@
       <c r="N37" s="10"/>
       <c r="O37" s="10"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="10"/>
       <c r="B38" s="10"/>
       <c r="C38" s="10"/>
@@ -2241,7 +2270,7 @@
       <c r="N38" s="10"/>
       <c r="O38" s="10"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="10"/>
       <c r="B39" s="10"/>
       <c r="C39" s="10"/>
@@ -2261,7 +2290,7 @@
       <c r="N39" s="10"/>
       <c r="O39" s="10"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="10"/>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
@@ -2281,7 +2310,7 @@
       <c r="N40" s="10"/>
       <c r="O40" s="10"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
       <c r="B41" s="10"/>
       <c r="C41" s="10"/>
@@ -2301,7 +2330,7 @@
       <c r="N41" s="10"/>
       <c r="O41" s="10"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="10"/>
       <c r="B42" s="10"/>
       <c r="C42" s="10"/>
@@ -2321,7 +2350,7 @@
       <c r="N42" s="10"/>
       <c r="O42" s="10"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
@@ -2341,7 +2370,7 @@
       <c r="N43" s="10"/>
       <c r="O43" s="10"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="10"/>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
@@ -2361,7 +2390,7 @@
       <c r="N44" s="10"/>
       <c r="O44" s="10"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="10"/>
       <c r="B45" s="10"/>
       <c r="C45" s="10"/>
@@ -2381,7 +2410,7 @@
       <c r="N45" s="10"/>
       <c r="O45" s="10"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="10"/>
       <c r="B46" s="10"/>
       <c r="C46" s="10"/>
@@ -2401,7 +2430,7 @@
       <c r="N46" s="10"/>
       <c r="O46" s="10"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
       <c r="C47" s="10"/>
@@ -2421,7 +2450,7 @@
       <c r="N47" s="10"/>
       <c r="O47" s="10"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="10"/>
       <c r="B48" s="10"/>
       <c r="C48" s="10"/>
@@ -2441,7 +2470,7 @@
       <c r="N48" s="10"/>
       <c r="O48" s="10"/>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="10"/>
       <c r="B49" s="10"/>
       <c r="C49" s="10"/>
@@ -2461,7 +2490,7 @@
       <c r="N49" s="10"/>
       <c r="O49" s="10"/>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="10"/>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
@@ -2481,7 +2510,7 @@
       <c r="N50" s="10"/>
       <c r="O50" s="10"/>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="10"/>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
@@ -2501,7 +2530,7 @@
       <c r="N51" s="10"/>
       <c r="O51" s="10"/>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="10"/>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
@@ -2521,7 +2550,7 @@
       <c r="N52" s="10"/>
       <c r="O52" s="10"/>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="10"/>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
@@ -2541,7 +2570,7 @@
       <c r="N53" s="10"/>
       <c r="O53" s="10"/>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="10"/>
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
@@ -2561,7 +2590,7 @@
       <c r="N54" s="10"/>
       <c r="O54" s="10"/>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="10"/>
       <c r="B55" s="10"/>
       <c r="C55" s="10"/>
@@ -2581,7 +2610,7 @@
       <c r="N55" s="10"/>
       <c r="O55" s="10"/>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="10"/>
       <c r="B56" s="10"/>
       <c r="C56" s="10"/>
@@ -2601,7 +2630,7 @@
       <c r="N56" s="10"/>
       <c r="O56" s="10"/>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="10"/>
       <c r="B57" s="10"/>
       <c r="C57" s="10"/>
@@ -2621,7 +2650,7 @@
       <c r="N57" s="10"/>
       <c r="O57" s="10"/>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="10"/>
       <c r="B58" s="10"/>
       <c r="C58" s="10"/>
@@ -2641,7 +2670,7 @@
       <c r="N58" s="10"/>
       <c r="O58" s="10"/>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="10"/>
       <c r="B59" s="10"/>
       <c r="C59" s="10"/>
@@ -2661,7 +2690,7 @@
       <c r="N59" s="10"/>
       <c r="O59" s="10"/>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="10"/>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
@@ -2681,7 +2710,7 @@
       <c r="N60" s="10"/>
       <c r="O60" s="10"/>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="10"/>
       <c r="B61" s="10"/>
       <c r="C61" s="10"/>
@@ -2701,7 +2730,7 @@
       <c r="N61" s="10"/>
       <c r="O61" s="10"/>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="10"/>
       <c r="B62" s="10"/>
       <c r="C62" s="10"/>
@@ -2721,7 +2750,7 @@
       <c r="N62" s="10"/>
       <c r="O62" s="10"/>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="10"/>
       <c r="B63" s="10"/>
       <c r="C63" s="10"/>
@@ -2741,7 +2770,7 @@
       <c r="N63" s="10"/>
       <c r="O63" s="10"/>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="10"/>
       <c r="B64" s="10"/>
       <c r="C64" s="10"/>
@@ -2761,7 +2790,7 @@
       <c r="N64" s="10"/>
       <c r="O64" s="10"/>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="10"/>
       <c r="B65" s="10"/>
       <c r="C65" s="10"/>
@@ -2781,7 +2810,7 @@
       <c r="N65" s="10"/>
       <c r="O65" s="10"/>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="10"/>
       <c r="B66" s="10"/>
       <c r="C66" s="10"/>
@@ -2801,7 +2830,7 @@
       <c r="N66" s="10"/>
       <c r="O66" s="10"/>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="10"/>
       <c r="B67" s="10"/>
       <c r="C67" s="10"/>
@@ -2821,7 +2850,7 @@
       <c r="N67" s="10"/>
       <c r="O67" s="10"/>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="10"/>
       <c r="B68" s="10"/>
       <c r="C68" s="10"/>
@@ -2841,7 +2870,7 @@
       <c r="N68" s="10"/>
       <c r="O68" s="10"/>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="10"/>
       <c r="B69" s="10"/>
       <c r="C69" s="10"/>
@@ -2861,7 +2890,7 @@
       <c r="N69" s="10"/>
       <c r="O69" s="10"/>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="10"/>
       <c r="B70" s="10"/>
       <c r="C70" s="10"/>
@@ -2881,7 +2910,7 @@
       <c r="N70" s="10"/>
       <c r="O70" s="10"/>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="10"/>
       <c r="B71" s="10"/>
       <c r="C71" s="10"/>
@@ -2901,7 +2930,7 @@
       <c r="N71" s="10"/>
       <c r="O71" s="10"/>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="10"/>
       <c r="B72" s="10"/>
       <c r="C72" s="10"/>
@@ -2921,7 +2950,7 @@
       <c r="N72" s="10"/>
       <c r="O72" s="10"/>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="10"/>
       <c r="B73" s="10"/>
       <c r="C73" s="10"/>
@@ -2941,7 +2970,7 @@
       <c r="N73" s="10"/>
       <c r="O73" s="10"/>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="10"/>
       <c r="B74" s="10"/>
       <c r="C74" s="10"/>
@@ -2961,7 +2990,7 @@
       <c r="N74" s="10"/>
       <c r="O74" s="10"/>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="10"/>
       <c r="B75" s="10"/>
       <c r="C75" s="10"/>
@@ -2981,7 +3010,7 @@
       <c r="N75" s="10"/>
       <c r="O75" s="10"/>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" s="10"/>
       <c r="B76" s="10"/>
       <c r="C76" s="10"/>
@@ -3001,7 +3030,7 @@
       <c r="N76" s="10"/>
       <c r="O76" s="10"/>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" s="10"/>
       <c r="B77" s="10"/>
       <c r="C77" s="10"/>
@@ -3021,7 +3050,7 @@
       <c r="N77" s="10"/>
       <c r="O77" s="10"/>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A78" s="10"/>
       <c r="B78" s="10"/>
       <c r="C78" s="10"/>
@@ -3041,7 +3070,7 @@
       <c r="N78" s="10"/>
       <c r="O78" s="10"/>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="10"/>
       <c r="B79" s="10"/>
       <c r="C79" s="10"/>
@@ -3061,7 +3090,7 @@
       <c r="N79" s="10"/>
       <c r="O79" s="10"/>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" s="10"/>
       <c r="B80" s="10"/>
       <c r="C80" s="10"/>
@@ -3081,7 +3110,7 @@
       <c r="N80" s="10"/>
       <c r="O80" s="10"/>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" s="10"/>
       <c r="B81" s="10"/>
       <c r="C81" s="10"/>
@@ -3101,7 +3130,7 @@
       <c r="N81" s="10"/>
       <c r="O81" s="10"/>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" s="10"/>
       <c r="B82" s="10"/>
       <c r="C82" s="10"/>
@@ -3121,7 +3150,7 @@
       <c r="N82" s="10"/>
       <c r="O82" s="10"/>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" s="10"/>
       <c r="B83" s="10"/>
       <c r="C83" s="10"/>
@@ -3141,7 +3170,7 @@
       <c r="N83" s="10"/>
       <c r="O83" s="10"/>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" s="10"/>
       <c r="B84" s="10"/>
       <c r="C84" s="10"/>
@@ -3161,7 +3190,7 @@
       <c r="N84" s="10"/>
       <c r="O84" s="10"/>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A85" s="10"/>
       <c r="B85" s="10"/>
       <c r="C85" s="10"/>
@@ -3181,7 +3210,7 @@
       <c r="N85" s="10"/>
       <c r="O85" s="10"/>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A86" s="10"/>
       <c r="B86" s="10"/>
       <c r="C86" s="10"/>
@@ -3201,7 +3230,7 @@
       <c r="N86" s="10"/>
       <c r="O86" s="10"/>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A87" s="10"/>
       <c r="B87" s="10"/>
       <c r="C87" s="10"/>
@@ -3221,7 +3250,7 @@
       <c r="N87" s="10"/>
       <c r="O87" s="10"/>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A88" s="10"/>
       <c r="B88" s="10"/>
       <c r="C88" s="10"/>
@@ -3241,7 +3270,7 @@
       <c r="N88" s="10"/>
       <c r="O88" s="10"/>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A89" s="10"/>
       <c r="B89" s="10"/>
       <c r="C89" s="10"/>
@@ -3261,7 +3290,7 @@
       <c r="N89" s="10"/>
       <c r="O89" s="10"/>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A90" s="10"/>
       <c r="B90" s="10"/>
       <c r="C90" s="10"/>
@@ -3281,7 +3310,7 @@
       <c r="N90" s="10"/>
       <c r="O90" s="10"/>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A91" s="10"/>
       <c r="B91" s="10"/>
       <c r="C91" s="10"/>
@@ -3301,7 +3330,7 @@
       <c r="N91" s="10"/>
       <c r="O91" s="10"/>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A92" s="10"/>
       <c r="B92" s="10"/>
       <c r="C92" s="10"/>
@@ -3321,7 +3350,7 @@
       <c r="N92" s="10"/>
       <c r="O92" s="10"/>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A93" s="10"/>
       <c r="B93" s="10"/>
       <c r="C93" s="10"/>
@@ -3341,7 +3370,7 @@
       <c r="N93" s="10"/>
       <c r="O93" s="10"/>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A94" s="10"/>
       <c r="B94" s="10"/>
       <c r="C94" s="10"/>
@@ -3361,7 +3390,7 @@
       <c r="N94" s="10"/>
       <c r="O94" s="10"/>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A95" s="10"/>
       <c r="B95" s="10"/>
       <c r="C95" s="10"/>
@@ -3381,7 +3410,7 @@
       <c r="N95" s="10"/>
       <c r="O95" s="10"/>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A96" s="10"/>
       <c r="B96" s="10"/>
       <c r="C96" s="10"/>
@@ -3401,7 +3430,7 @@
       <c r="N96" s="10"/>
       <c r="O96" s="10"/>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A97" s="10"/>
       <c r="B97" s="10"/>
       <c r="C97" s="10"/>
@@ -3421,7 +3450,7 @@
       <c r="N97" s="10"/>
       <c r="O97" s="10"/>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A98" s="10"/>
       <c r="B98" s="10"/>
       <c r="C98" s="10"/>
@@ -3441,7 +3470,7 @@
       <c r="N98" s="10"/>
       <c r="O98" s="10"/>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A99" s="10"/>
       <c r="B99" s="10"/>
       <c r="C99" s="10"/>
@@ -3461,7 +3490,7 @@
       <c r="N99" s="10"/>
       <c r="O99" s="10"/>
     </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A100" s="10"/>
       <c r="B100" s="10"/>
       <c r="C100" s="10"/>
@@ -3481,7 +3510,7 @@
       <c r="N100" s="10"/>
       <c r="O100" s="10"/>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A101" s="10"/>
       <c r="B101" s="10"/>
       <c r="C101" s="10"/>
@@ -3501,7 +3530,7 @@
       <c r="N101" s="10"/>
       <c r="O101" s="10"/>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A102" s="10"/>
       <c r="B102" s="10"/>
       <c r="C102" s="10"/>
@@ -3521,7 +3550,7 @@
       <c r="N102" s="10"/>
       <c r="O102" s="10"/>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A103" s="10"/>
       <c r="B103" s="10"/>
       <c r="C103" s="10"/>
@@ -3541,7 +3570,7 @@
       <c r="N103" s="10"/>
       <c r="O103" s="10"/>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A104" s="10"/>
       <c r="B104" s="10"/>
       <c r="C104" s="10"/>
@@ -3561,7 +3590,7 @@
       <c r="N104" s="10"/>
       <c r="O104" s="10"/>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A105" s="10"/>
       <c r="B105" s="10"/>
       <c r="C105" s="10"/>
@@ -3581,7 +3610,7 @@
       <c r="N105" s="10"/>
       <c r="O105" s="10"/>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A106" s="10"/>
       <c r="B106" s="10"/>
       <c r="C106" s="10"/>
@@ -3601,7 +3630,7 @@
       <c r="N106" s="10"/>
       <c r="O106" s="10"/>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A107" s="10"/>
       <c r="B107" s="10"/>
       <c r="C107" s="10"/>
@@ -3621,7 +3650,7 @@
       <c r="N107" s="10"/>
       <c r="O107" s="10"/>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A108" s="10"/>
       <c r="B108" s="10"/>
       <c r="C108" s="10"/>
@@ -3641,7 +3670,7 @@
       <c r="N108" s="10"/>
       <c r="O108" s="10"/>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A109" s="10"/>
       <c r="B109" s="10"/>
       <c r="C109" s="10"/>
@@ -3661,7 +3690,7 @@
       <c r="N109" s="10"/>
       <c r="O109" s="10"/>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A110" s="10"/>
       <c r="B110" s="10"/>
       <c r="C110" s="10"/>
@@ -3681,7 +3710,7 @@
       <c r="N110" s="10"/>
       <c r="O110" s="10"/>
     </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A111" s="10"/>
       <c r="B111" s="10"/>
       <c r="C111" s="10"/>
@@ -3701,7 +3730,7 @@
       <c r="N111" s="10"/>
       <c r="O111" s="10"/>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A112" s="10"/>
       <c r="B112" s="10"/>
       <c r="C112" s="10"/>
@@ -3721,7 +3750,7 @@
       <c r="N112" s="10"/>
       <c r="O112" s="10"/>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A113" s="10"/>
       <c r="B113" s="10"/>
       <c r="C113" s="10"/>
@@ -3741,7 +3770,7 @@
       <c r="N113" s="10"/>
       <c r="O113" s="10"/>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A114" s="10"/>
       <c r="B114" s="10"/>
       <c r="C114" s="10"/>
@@ -3761,7 +3790,7 @@
       <c r="N114" s="10"/>
       <c r="O114" s="10"/>
     </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A115" s="10"/>
       <c r="B115" s="10"/>
       <c r="C115" s="10"/>
@@ -3781,7 +3810,7 @@
       <c r="N115" s="10"/>
       <c r="O115" s="10"/>
     </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A116" s="10"/>
       <c r="B116" s="10"/>
       <c r="C116" s="10"/>
@@ -3801,7 +3830,7 @@
       <c r="N116" s="10"/>
       <c r="O116" s="10"/>
     </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A117" s="10"/>
       <c r="B117" s="10"/>
       <c r="C117" s="10"/>
@@ -3821,7 +3850,7 @@
       <c r="N117" s="10"/>
       <c r="O117" s="10"/>
     </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A118" s="10"/>
       <c r="B118" s="10"/>
       <c r="C118" s="10"/>
@@ -3841,7 +3870,7 @@
       <c r="N118" s="10"/>
       <c r="O118" s="10"/>
     </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A119" s="10"/>
       <c r="B119" s="10"/>
       <c r="C119" s="10"/>
@@ -3861,7 +3890,7 @@
       <c r="N119" s="10"/>
       <c r="O119" s="10"/>
     </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A120" s="10"/>
       <c r="B120" s="10"/>
       <c r="C120" s="10"/>
@@ -3881,7 +3910,7 @@
       <c r="N120" s="10"/>
       <c r="O120" s="10"/>
     </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A121" s="10"/>
       <c r="B121" s="10"/>
       <c r="C121" s="10"/>
@@ -3901,7 +3930,7 @@
       <c r="N121" s="10"/>
       <c r="O121" s="10"/>
     </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A122" s="10"/>
       <c r="B122" s="10"/>
       <c r="C122" s="10"/>
@@ -3921,7 +3950,7 @@
       <c r="N122" s="10"/>
       <c r="O122" s="10"/>
     </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A123" s="10"/>
       <c r="B123" s="10"/>
       <c r="C123" s="10"/>
@@ -3941,7 +3970,7 @@
       <c r="N123" s="10"/>
       <c r="O123" s="10"/>
     </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A124" s="10"/>
       <c r="B124" s="10"/>
       <c r="C124" s="10"/>
@@ -3961,7 +3990,7 @@
       <c r="N124" s="10"/>
       <c r="O124" s="10"/>
     </row>
-    <row r="125" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A125" s="10"/>
       <c r="B125" s="10"/>
       <c r="C125" s="10"/>
@@ -3981,7 +4010,7 @@
       <c r="N125" s="10"/>
       <c r="O125" s="10"/>
     </row>
-    <row r="126" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A126" s="10"/>
       <c r="B126" s="10"/>
       <c r="C126" s="10"/>
@@ -4001,7 +4030,7 @@
       <c r="N126" s="10"/>
       <c r="O126" s="10"/>
     </row>
-    <row r="127" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A127" s="10"/>
       <c r="B127" s="10"/>
       <c r="C127" s="10"/>
@@ -4021,7 +4050,7 @@
       <c r="N127" s="10"/>
       <c r="O127" s="10"/>
     </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A128" s="10"/>
       <c r="B128" s="10"/>
       <c r="C128" s="10"/>
@@ -4041,7 +4070,7 @@
       <c r="N128" s="10"/>
       <c r="O128" s="10"/>
     </row>
-    <row r="129" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A129" s="10"/>
       <c r="B129" s="10"/>
       <c r="C129" s="10"/>
@@ -4061,7 +4090,7 @@
       <c r="N129" s="10"/>
       <c r="O129" s="10"/>
     </row>
-    <row r="130" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A130" s="10"/>
       <c r="B130" s="10"/>
       <c r="C130" s="10"/>
@@ -4081,7 +4110,7 @@
       <c r="N130" s="10"/>
       <c r="O130" s="10"/>
     </row>
-    <row r="131" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A131" s="10"/>
       <c r="B131" s="10"/>
       <c r="C131" s="10"/>
@@ -4101,7 +4130,7 @@
       <c r="N131" s="10"/>
       <c r="O131" s="10"/>
     </row>
-    <row r="132" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A132" s="10"/>
       <c r="B132" s="10"/>
       <c r="C132" s="10"/>
@@ -4121,7 +4150,7 @@
       <c r="N132" s="10"/>
       <c r="O132" s="10"/>
     </row>
-    <row r="133" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A133" s="10"/>
       <c r="B133" s="10"/>
       <c r="C133" s="10"/>
@@ -4141,7 +4170,7 @@
       <c r="N133" s="10"/>
       <c r="O133" s="10"/>
     </row>
-    <row r="134" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A134" s="10"/>
       <c r="B134" s="10"/>
       <c r="C134" s="10"/>
@@ -4161,7 +4190,7 @@
       <c r="N134" s="10"/>
       <c r="O134" s="10"/>
     </row>
-    <row r="135" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A135" s="10"/>
       <c r="B135" s="10"/>
       <c r="C135" s="10"/>
@@ -4181,7 +4210,7 @@
       <c r="N135" s="10"/>
       <c r="O135" s="10"/>
     </row>
-    <row r="136" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A136" s="10"/>
       <c r="B136" s="10"/>
       <c r="C136" s="10"/>
@@ -4201,7 +4230,7 @@
       <c r="N136" s="10"/>
       <c r="O136" s="10"/>
     </row>
-    <row r="137" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A137" s="10"/>
       <c r="B137" s="10"/>
       <c r="C137" s="10"/>
@@ -4221,7 +4250,7 @@
       <c r="N137" s="10"/>
       <c r="O137" s="10"/>
     </row>
-    <row r="138" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A138" s="10"/>
       <c r="B138" s="10"/>
       <c r="C138" s="10"/>
@@ -4241,7 +4270,7 @@
       <c r="N138" s="10"/>
       <c r="O138" s="10"/>
     </row>
-    <row r="139" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A139" s="10"/>
       <c r="B139" s="10"/>
       <c r="C139" s="10"/>
@@ -4261,7 +4290,7 @@
       <c r="N139" s="10"/>
       <c r="O139" s="10"/>
     </row>
-    <row r="140" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A140" s="10"/>
       <c r="B140" s="10"/>
       <c r="C140" s="10"/>
@@ -4281,7 +4310,7 @@
       <c r="N140" s="10"/>
       <c r="O140" s="10"/>
     </row>
-    <row r="141" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A141" s="10"/>
       <c r="B141" s="10"/>
       <c r="C141" s="10"/>
@@ -4301,7 +4330,7 @@
       <c r="N141" s="10"/>
       <c r="O141" s="10"/>
     </row>
-    <row r="142" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A142" s="10"/>
       <c r="B142" s="10"/>
       <c r="C142" s="10"/>
@@ -4321,7 +4350,7 @@
       <c r="N142" s="10"/>
       <c r="O142" s="10"/>
     </row>
-    <row r="143" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A143" s="10"/>
       <c r="B143" s="10"/>
       <c r="C143" s="10"/>
@@ -4341,7 +4370,7 @@
       <c r="N143" s="10"/>
       <c r="O143" s="10"/>
     </row>
-    <row r="144" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A144" s="10"/>
       <c r="B144" s="10"/>
       <c r="C144" s="10"/>
@@ -4361,7 +4390,7 @@
       <c r="N144" s="10"/>
       <c r="O144" s="10"/>
     </row>
-    <row r="145" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A145" s="10"/>
       <c r="B145" s="10"/>
       <c r="C145" s="10"/>
@@ -4381,7 +4410,7 @@
       <c r="N145" s="10"/>
       <c r="O145" s="10"/>
     </row>
-    <row r="146" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A146" s="10"/>
       <c r="B146" s="10"/>
       <c r="C146" s="10"/>
@@ -4401,7 +4430,7 @@
       <c r="N146" s="10"/>
       <c r="O146" s="10"/>
     </row>
-    <row r="147" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A147" s="10"/>
       <c r="B147" s="10"/>
       <c r="C147" s="10"/>
@@ -4421,7 +4450,7 @@
       <c r="N147" s="10"/>
       <c r="O147" s="10"/>
     </row>
-    <row r="148" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A148" s="10"/>
       <c r="B148" s="10"/>
       <c r="C148" s="10"/>
@@ -4441,7 +4470,7 @@
       <c r="N148" s="10"/>
       <c r="O148" s="10"/>
     </row>
-    <row r="149" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A149" s="10"/>
       <c r="B149" s="10"/>
       <c r="C149" s="10"/>
@@ -4461,7 +4490,7 @@
       <c r="N149" s="10"/>
       <c r="O149" s="10"/>
     </row>
-    <row r="150" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A150" s="10"/>
       <c r="B150" s="10"/>
       <c r="C150" s="10"/>
@@ -4481,7 +4510,7 @@
       <c r="N150" s="10"/>
       <c r="O150" s="10"/>
     </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A151" s="10"/>
       <c r="B151" s="10"/>
       <c r="C151" s="10"/>
@@ -4501,7 +4530,7 @@
       <c r="N151" s="10"/>
       <c r="O151" s="10"/>
     </row>
-    <row r="152" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A152" s="10"/>
       <c r="B152" s="10"/>
       <c r="C152" s="10"/>
@@ -4521,7 +4550,7 @@
       <c r="N152" s="10"/>
       <c r="O152" s="10"/>
     </row>
-    <row r="153" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A153" s="10"/>
       <c r="B153" s="10"/>
       <c r="C153" s="10"/>
@@ -4541,7 +4570,7 @@
       <c r="N153" s="10"/>
       <c r="O153" s="10"/>
     </row>
-    <row r="154" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A154" s="10"/>
       <c r="B154" s="10"/>
       <c r="C154" s="10"/>
@@ -4561,7 +4590,7 @@
       <c r="N154" s="10"/>
       <c r="O154" s="10"/>
     </row>
-    <row r="155" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A155" s="10"/>
       <c r="B155" s="10"/>
       <c r="C155" s="10"/>
@@ -4581,7 +4610,7 @@
       <c r="N155" s="10"/>
       <c r="O155" s="10"/>
     </row>
-    <row r="156" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A156" s="10"/>
       <c r="B156" s="10"/>
       <c r="C156" s="10"/>
@@ -4601,7 +4630,7 @@
       <c r="N156" s="10"/>
       <c r="O156" s="10"/>
     </row>
-    <row r="157" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A157" s="10"/>
       <c r="B157" s="10"/>
       <c r="C157" s="10"/>
@@ -4621,7 +4650,7 @@
       <c r="N157" s="10"/>
       <c r="O157" s="10"/>
     </row>
-    <row r="158" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A158" s="10"/>
       <c r="B158" s="10"/>
       <c r="C158" s="10"/>
@@ -4641,7 +4670,7 @@
       <c r="N158" s="10"/>
       <c r="O158" s="10"/>
     </row>
-    <row r="159" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A159" s="10"/>
       <c r="B159" s="10"/>
       <c r="C159" s="10"/>
@@ -4661,7 +4690,7 @@
       <c r="N159" s="10"/>
       <c r="O159" s="10"/>
     </row>
-    <row r="160" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A160" s="10"/>
       <c r="B160" s="10"/>
       <c r="C160" s="10"/>
@@ -4681,7 +4710,7 @@
       <c r="N160" s="10"/>
       <c r="O160" s="10"/>
     </row>
-    <row r="161" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A161" s="10"/>
       <c r="B161" s="10"/>
       <c r="C161" s="10"/>
@@ -4701,7 +4730,7 @@
       <c r="N161" s="10"/>
       <c r="O161" s="10"/>
     </row>
-    <row r="162" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A162" s="10"/>
       <c r="B162" s="10"/>
       <c r="C162" s="10"/>
@@ -4721,7 +4750,7 @@
       <c r="N162" s="10"/>
       <c r="O162" s="10"/>
     </row>
-    <row r="163" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A163" s="10"/>
       <c r="B163" s="10"/>
       <c r="C163" s="10"/>
@@ -4741,7 +4770,7 @@
       <c r="N163" s="10"/>
       <c r="O163" s="10"/>
     </row>
-    <row r="164" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A164" s="10"/>
       <c r="B164" s="10"/>
       <c r="C164" s="10"/>
@@ -4761,7 +4790,7 @@
       <c r="N164" s="10"/>
       <c r="O164" s="10"/>
     </row>
-    <row r="165" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A165" s="10"/>
       <c r="B165" s="10"/>
       <c r="C165" s="10"/>
@@ -4781,7 +4810,7 @@
       <c r="N165" s="10"/>
       <c r="O165" s="10"/>
     </row>
-    <row r="166" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A166" s="10"/>
       <c r="B166" s="10"/>
       <c r="C166" s="10"/>
@@ -4801,7 +4830,7 @@
       <c r="N166" s="10"/>
       <c r="O166" s="10"/>
     </row>
-    <row r="167" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A167" s="10"/>
       <c r="B167" s="10"/>
       <c r="C167" s="10"/>
@@ -4821,7 +4850,7 @@
       <c r="N167" s="10"/>
       <c r="O167" s="10"/>
     </row>
-    <row r="168" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A168" s="10"/>
       <c r="B168" s="10"/>
       <c r="C168" s="10"/>
@@ -4841,7 +4870,7 @@
       <c r="N168" s="10"/>
       <c r="O168" s="10"/>
     </row>
-    <row r="169" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A169" s="10"/>
       <c r="B169" s="10"/>
       <c r="C169" s="10"/>
@@ -4861,7 +4890,7 @@
       <c r="N169" s="10"/>
       <c r="O169" s="10"/>
     </row>
-    <row r="170" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A170" s="10"/>
       <c r="B170" s="10"/>
       <c r="C170" s="10"/>
@@ -4881,7 +4910,7 @@
       <c r="N170" s="10"/>
       <c r="O170" s="10"/>
     </row>
-    <row r="171" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A171" s="10"/>
       <c r="B171" s="10"/>
       <c r="C171" s="10"/>
@@ -4901,7 +4930,7 @@
       <c r="N171" s="10"/>
       <c r="O171" s="10"/>
     </row>
-    <row r="172" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A172" s="10"/>
       <c r="B172" s="10"/>
       <c r="C172" s="10"/>
@@ -4921,7 +4950,7 @@
       <c r="N172" s="10"/>
       <c r="O172" s="10"/>
     </row>
-    <row r="173" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A173" s="10"/>
       <c r="B173" s="10"/>
       <c r="C173" s="10"/>
@@ -4941,7 +4970,7 @@
       <c r="N173" s="10"/>
       <c r="O173" s="10"/>
     </row>
-    <row r="174" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A174" s="10"/>
       <c r="B174" s="10"/>
       <c r="C174" s="10"/>
@@ -4961,7 +4990,7 @@
       <c r="N174" s="10"/>
       <c r="O174" s="10"/>
     </row>
-    <row r="175" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A175" s="10"/>
       <c r="B175" s="10"/>
       <c r="C175" s="10"/>
@@ -4981,7 +5010,7 @@
       <c r="N175" s="10"/>
       <c r="O175" s="10"/>
     </row>
-    <row r="176" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A176" s="10"/>
       <c r="B176" s="10"/>
       <c r="C176" s="10"/>
@@ -5001,7 +5030,7 @@
       <c r="N176" s="10"/>
       <c r="O176" s="10"/>
     </row>
-    <row r="177" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A177" s="10"/>
       <c r="B177" s="10"/>
       <c r="C177" s="10"/>
@@ -5021,7 +5050,7 @@
       <c r="N177" s="10"/>
       <c r="O177" s="10"/>
     </row>
-    <row r="178" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A178" s="10"/>
       <c r="B178" s="10"/>
       <c r="C178" s="10"/>
@@ -5041,7 +5070,7 @@
       <c r="N178" s="10"/>
       <c r="O178" s="10"/>
     </row>
-    <row r="179" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A179" s="10"/>
       <c r="B179" s="10"/>
       <c r="C179" s="10"/>
@@ -5061,7 +5090,7 @@
       <c r="N179" s="10"/>
       <c r="O179" s="10"/>
     </row>
-    <row r="180" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A180" s="10"/>
       <c r="B180" s="10"/>
       <c r="C180" s="10"/>
@@ -5081,7 +5110,7 @@
       <c r="N180" s="10"/>
       <c r="O180" s="10"/>
     </row>
-    <row r="181" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A181" s="10"/>
       <c r="B181" s="10"/>
       <c r="C181" s="10"/>
@@ -5101,7 +5130,7 @@
       <c r="N181" s="10"/>
       <c r="O181" s="10"/>
     </row>
-    <row r="182" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A182" s="10"/>
       <c r="B182" s="10"/>
       <c r="C182" s="10"/>
@@ -5121,7 +5150,7 @@
       <c r="N182" s="10"/>
       <c r="O182" s="10"/>
     </row>
-    <row r="183" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A183" s="10"/>
       <c r="B183" s="10"/>
       <c r="C183" s="10"/>
@@ -5141,7 +5170,7 @@
       <c r="N183" s="10"/>
       <c r="O183" s="10"/>
     </row>
-    <row r="184" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A184" s="10"/>
       <c r="B184" s="10"/>
       <c r="C184" s="10"/>
@@ -5161,7 +5190,7 @@
       <c r="N184" s="10"/>
       <c r="O184" s="10"/>
     </row>
-    <row r="185" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A185" s="10"/>
       <c r="B185" s="10"/>
       <c r="C185" s="10"/>
@@ -5181,7 +5210,7 @@
       <c r="N185" s="10"/>
       <c r="O185" s="10"/>
     </row>
-    <row r="186" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A186" s="10"/>
       <c r="B186" s="10"/>
       <c r="C186" s="10"/>
@@ -5201,7 +5230,7 @@
       <c r="N186" s="10"/>
       <c r="O186" s="10"/>
     </row>
-    <row r="187" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A187" s="10"/>
       <c r="B187" s="10"/>
       <c r="C187" s="10"/>
@@ -5221,7 +5250,7 @@
       <c r="N187" s="10"/>
       <c r="O187" s="10"/>
     </row>
-    <row r="188" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A188" s="10"/>
       <c r="B188" s="10"/>
       <c r="C188" s="10"/>
@@ -5241,7 +5270,7 @@
       <c r="N188" s="10"/>
       <c r="O188" s="10"/>
     </row>
-    <row r="189" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A189" s="10"/>
       <c r="B189" s="10"/>
       <c r="C189" s="10"/>
@@ -5261,7 +5290,7 @@
       <c r="N189" s="10"/>
       <c r="O189" s="10"/>
     </row>
-    <row r="190" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A190" s="10"/>
       <c r="B190" s="10"/>
       <c r="C190" s="10"/>
@@ -5281,7 +5310,7 @@
       <c r="N190" s="10"/>
       <c r="O190" s="10"/>
     </row>
-    <row r="191" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A191" s="10"/>
       <c r="B191" s="10"/>
       <c r="C191" s="10"/>
@@ -5301,7 +5330,7 @@
       <c r="N191" s="10"/>
       <c r="O191" s="10"/>
     </row>
-    <row r="192" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A192" s="10"/>
       <c r="B192" s="10"/>
       <c r="C192" s="10"/>
@@ -5321,7 +5350,7 @@
       <c r="N192" s="10"/>
       <c r="O192" s="10"/>
     </row>
-    <row r="193" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A193" s="10"/>
       <c r="B193" s="10"/>
       <c r="C193" s="10"/>
@@ -5341,7 +5370,7 @@
       <c r="N193" s="10"/>
       <c r="O193" s="10"/>
     </row>
-    <row r="194" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A194" s="10"/>
       <c r="B194" s="10"/>
       <c r="C194" s="10"/>
@@ -5361,7 +5390,7 @@
       <c r="N194" s="10"/>
       <c r="O194" s="10"/>
     </row>
-    <row r="195" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A195" s="10"/>
       <c r="B195" s="10"/>
       <c r="C195" s="10"/>
@@ -5381,7 +5410,7 @@
       <c r="N195" s="10"/>
       <c r="O195" s="10"/>
     </row>
-    <row r="196" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A196" s="10"/>
       <c r="B196" s="10"/>
       <c r="C196" s="10"/>
@@ -5401,7 +5430,7 @@
       <c r="N196" s="10"/>
       <c r="O196" s="10"/>
     </row>
-    <row r="197" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A197" s="10"/>
       <c r="B197" s="10"/>
       <c r="C197" s="10"/>
@@ -5421,7 +5450,7 @@
       <c r="N197" s="10"/>
       <c r="O197" s="10"/>
     </row>
-    <row r="198" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A198" s="10"/>
       <c r="B198" s="10"/>
       <c r="C198" s="10"/>
@@ -5441,7 +5470,7 @@
       <c r="N198" s="10"/>
       <c r="O198" s="10"/>
     </row>
-    <row r="199" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A199" s="10"/>
       <c r="B199" s="10"/>
       <c r="C199" s="10"/>
@@ -5461,7 +5490,7 @@
       <c r="N199" s="10"/>
       <c r="O199" s="10"/>
     </row>
-    <row r="200" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A200" s="10"/>
       <c r="B200" s="10"/>
       <c r="C200" s="10"/>
@@ -5481,7 +5510,7 @@
       <c r="N200" s="10"/>
       <c r="O200" s="10"/>
     </row>
-    <row r="201" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A201" s="10"/>
       <c r="B201" s="10"/>
       <c r="C201" s="10"/>
@@ -5501,7 +5530,7 @@
       <c r="N201" s="10"/>
       <c r="O201" s="10"/>
     </row>
-    <row r="202" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A202" s="10"/>
       <c r="B202" s="10"/>
       <c r="C202" s="10"/>
@@ -5521,7 +5550,7 @@
       <c r="N202" s="10"/>
       <c r="O202" s="10"/>
     </row>
-    <row r="203" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A203" s="10"/>
       <c r="B203" s="10"/>
       <c r="C203" s="10"/>
@@ -5541,7 +5570,7 @@
       <c r="N203" s="10"/>
       <c r="O203" s="10"/>
     </row>
-    <row r="204" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A204" s="10"/>
       <c r="B204" s="10"/>
       <c r="C204" s="10"/>
@@ -5561,7 +5590,7 @@
       <c r="N204" s="10"/>
       <c r="O204" s="10"/>
     </row>
-    <row r="205" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A205" s="10"/>
       <c r="B205" s="10"/>
       <c r="C205" s="10"/>
@@ -5581,7 +5610,7 @@
       <c r="N205" s="10"/>
       <c r="O205" s="10"/>
     </row>
-    <row r="206" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A206" s="10"/>
       <c r="B206" s="10"/>
       <c r="C206" s="10"/>
@@ -5601,7 +5630,7 @@
       <c r="N206" s="10"/>
       <c r="O206" s="10"/>
     </row>
-    <row r="207" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A207" s="10"/>
       <c r="B207" s="10"/>
       <c r="C207" s="10"/>
@@ -5621,7 +5650,7 @@
       <c r="N207" s="10"/>
       <c r="O207" s="10"/>
     </row>
-    <row r="208" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A208" s="10"/>
       <c r="B208" s="10"/>
       <c r="C208" s="10"/>
@@ -5641,7 +5670,7 @@
       <c r="N208" s="10"/>
       <c r="O208" s="10"/>
     </row>
-    <row r="209" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A209" s="10"/>
       <c r="B209" s="10"/>
       <c r="C209" s="10"/>
@@ -5661,7 +5690,7 @@
       <c r="N209" s="10"/>
       <c r="O209" s="10"/>
     </row>
-    <row r="210" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A210" s="10"/>
       <c r="B210" s="10"/>
       <c r="C210" s="10"/>
@@ -5681,7 +5710,7 @@
       <c r="N210" s="10"/>
       <c r="O210" s="10"/>
     </row>
-    <row r="211" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A211" s="10"/>
       <c r="B211" s="10"/>
       <c r="C211" s="10"/>
@@ -5701,7 +5730,7 @@
       <c r="N211" s="10"/>
       <c r="O211" s="10"/>
     </row>
-    <row r="212" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A212" s="10"/>
       <c r="B212" s="10"/>
       <c r="C212" s="10"/>
@@ -5721,7 +5750,7 @@
       <c r="N212" s="10"/>
       <c r="O212" s="10"/>
     </row>
-    <row r="213" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A213" s="10"/>
       <c r="B213" s="10"/>
       <c r="C213" s="10"/>
@@ -5741,7 +5770,7 @@
       <c r="N213" s="10"/>
       <c r="O213" s="10"/>
     </row>
-    <row r="214" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A214" s="10"/>
       <c r="B214" s="10"/>
       <c r="C214" s="10"/>
@@ -5761,7 +5790,7 @@
       <c r="N214" s="10"/>
       <c r="O214" s="10"/>
     </row>
-    <row r="215" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A215" s="10"/>
       <c r="B215" s="10"/>
       <c r="C215" s="10"/>
@@ -5781,7 +5810,7 @@
       <c r="N215" s="10"/>
       <c r="O215" s="10"/>
     </row>
-    <row r="216" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A216" s="10"/>
       <c r="B216" s="10"/>
       <c r="C216" s="10"/>
@@ -5801,7 +5830,7 @@
       <c r="N216" s="10"/>
       <c r="O216" s="10"/>
     </row>
-    <row r="217" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A217" s="10"/>
       <c r="B217" s="10"/>
       <c r="C217" s="10"/>
@@ -5821,7 +5850,7 @@
       <c r="N217" s="10"/>
       <c r="O217" s="10"/>
     </row>
-    <row r="218" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A218" s="10"/>
       <c r="B218" s="10"/>
       <c r="C218" s="10"/>
@@ -5841,7 +5870,7 @@
       <c r="N218" s="10"/>
       <c r="O218" s="10"/>
     </row>
-    <row r="219" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A219" s="10"/>
       <c r="B219" s="10"/>
       <c r="C219" s="10"/>
@@ -5861,7 +5890,7 @@
       <c r="N219" s="10"/>
       <c r="O219" s="10"/>
     </row>
-    <row r="220" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A220" s="10"/>
       <c r="B220" s="10"/>
       <c r="C220" s="10"/>
@@ -5881,7 +5910,7 @@
       <c r="N220" s="10"/>
       <c r="O220" s="10"/>
     </row>
-    <row r="221" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A221" s="10"/>
       <c r="B221" s="10"/>
       <c r="C221" s="10"/>
@@ -5901,7 +5930,7 @@
       <c r="N221" s="10"/>
       <c r="O221" s="10"/>
     </row>
-    <row r="222" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A222" s="10"/>
       <c r="B222" s="10"/>
       <c r="C222" s="10"/>
@@ -5921,7 +5950,7 @@
       <c r="N222" s="10"/>
       <c r="O222" s="10"/>
     </row>
-    <row r="223" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A223" s="10"/>
       <c r="B223" s="10"/>
       <c r="C223" s="10"/>
@@ -5941,7 +5970,7 @@
       <c r="N223" s="10"/>
       <c r="O223" s="10"/>
     </row>
-    <row r="224" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A224" s="10"/>
       <c r="B224" s="10"/>
       <c r="C224" s="10"/>
@@ -5961,7 +5990,7 @@
       <c r="N224" s="10"/>
       <c r="O224" s="10"/>
     </row>
-    <row r="225" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A225" s="10"/>
       <c r="B225" s="10"/>
       <c r="C225" s="10"/>
@@ -5981,7 +6010,7 @@
       <c r="N225" s="10"/>
       <c r="O225" s="10"/>
     </row>
-    <row r="226" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A226" s="10"/>
       <c r="B226" s="10"/>
       <c r="C226" s="10"/>
@@ -6001,7 +6030,7 @@
       <c r="N226" s="10"/>
       <c r="O226" s="10"/>
     </row>
-    <row r="227" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A227" s="10"/>
       <c r="B227" s="10"/>
       <c r="C227" s="10"/>
@@ -6021,7 +6050,7 @@
       <c r="N227" s="10"/>
       <c r="O227" s="10"/>
     </row>
-    <row r="228" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A228" s="10"/>
       <c r="B228" s="10"/>
       <c r="C228" s="10"/>
@@ -6041,7 +6070,7 @@
       <c r="N228" s="10"/>
       <c r="O228" s="10"/>
     </row>
-    <row r="229" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A229" s="10"/>
       <c r="B229" s="10"/>
       <c r="C229" s="10"/>
@@ -6061,7 +6090,7 @@
       <c r="N229" s="10"/>
       <c r="O229" s="10"/>
     </row>
-    <row r="230" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A230" s="10"/>
       <c r="B230" s="10"/>
       <c r="C230" s="10"/>
@@ -6081,7 +6110,7 @@
       <c r="N230" s="10"/>
       <c r="O230" s="10"/>
     </row>
-    <row r="231" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A231" s="10"/>
       <c r="B231" s="10"/>
       <c r="C231" s="10"/>
@@ -6101,7 +6130,7 @@
       <c r="N231" s="10"/>
       <c r="O231" s="10"/>
     </row>
-    <row r="232" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A232" s="10"/>
       <c r="B232" s="10"/>
       <c r="C232" s="10"/>
@@ -6121,7 +6150,7 @@
       <c r="N232" s="10"/>
       <c r="O232" s="10"/>
     </row>
-    <row r="233" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A233" s="10"/>
       <c r="B233" s="10"/>
       <c r="C233" s="10"/>
@@ -6141,7 +6170,7 @@
       <c r="N233" s="10"/>
       <c r="O233" s="10"/>
     </row>
-    <row r="234" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A234" s="10"/>
       <c r="B234" s="10"/>
       <c r="C234" s="10"/>
@@ -6161,7 +6190,7 @@
       <c r="N234" s="10"/>
       <c r="O234" s="10"/>
     </row>
-    <row r="235" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A235" s="10"/>
       <c r="B235" s="10"/>
       <c r="C235" s="10"/>
@@ -6181,7 +6210,7 @@
       <c r="N235" s="10"/>
       <c r="O235" s="10"/>
     </row>
-    <row r="236" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A236" s="10"/>
       <c r="B236" s="10"/>
       <c r="C236" s="10"/>
@@ -6201,7 +6230,7 @@
       <c r="N236" s="10"/>
       <c r="O236" s="10"/>
     </row>
-    <row r="237" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A237" s="10"/>
       <c r="B237" s="10"/>
       <c r="C237" s="10"/>
@@ -6221,7 +6250,7 @@
       <c r="N237" s="10"/>
       <c r="O237" s="10"/>
     </row>
-    <row r="238" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A238" s="10"/>
       <c r="B238" s="10"/>
       <c r="C238" s="10"/>
@@ -6241,7 +6270,7 @@
       <c r="N238" s="10"/>
       <c r="O238" s="10"/>
     </row>
-    <row r="239" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A239" s="10"/>
       <c r="B239" s="10"/>
       <c r="C239" s="10"/>
@@ -6261,7 +6290,7 @@
       <c r="N239" s="10"/>
       <c r="O239" s="10"/>
     </row>
-    <row r="240" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A240" s="10"/>
       <c r="B240" s="10"/>
       <c r="C240" s="10"/>
@@ -6281,7 +6310,7 @@
       <c r="N240" s="10"/>
       <c r="O240" s="10"/>
     </row>
-    <row r="241" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A241" s="10"/>
       <c r="B241" s="10"/>
       <c r="C241" s="10"/>
@@ -6301,7 +6330,7 @@
       <c r="N241" s="10"/>
       <c r="O241" s="10"/>
     </row>
-    <row r="242" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A242" s="10"/>
       <c r="B242" s="10"/>
       <c r="C242" s="10"/>
@@ -6321,7 +6350,7 @@
       <c r="N242" s="10"/>
       <c r="O242" s="10"/>
     </row>
-    <row r="243" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A243" s="10"/>
       <c r="B243" s="10"/>
       <c r="C243" s="10"/>
@@ -6341,7 +6370,7 @@
       <c r="N243" s="10"/>
       <c r="O243" s="10"/>
     </row>
-    <row r="244" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A244" s="10"/>
       <c r="B244" s="10"/>
       <c r="C244" s="10"/>
@@ -6361,7 +6390,7 @@
       <c r="N244" s="10"/>
       <c r="O244" s="10"/>
     </row>
-    <row r="245" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A245" s="10"/>
       <c r="B245" s="10"/>
       <c r="C245" s="10"/>
@@ -6381,7 +6410,7 @@
       <c r="N245" s="10"/>
       <c r="O245" s="10"/>
     </row>
-    <row r="246" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A246" s="10"/>
       <c r="B246" s="10"/>
       <c r="C246" s="10"/>
@@ -6401,7 +6430,7 @@
       <c r="N246" s="10"/>
       <c r="O246" s="10"/>
     </row>
-    <row r="247" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A247" s="10"/>
       <c r="B247" s="10"/>
       <c r="C247" s="10"/>
@@ -6421,7 +6450,7 @@
       <c r="N247" s="10"/>
       <c r="O247" s="10"/>
     </row>
-    <row r="248" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A248" s="10"/>
       <c r="B248" s="10"/>
       <c r="C248" s="10"/>
@@ -6441,7 +6470,7 @@
       <c r="N248" s="10"/>
       <c r="O248" s="10"/>
     </row>
-    <row r="249" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A249" s="10"/>
       <c r="B249" s="10"/>
       <c r="C249" s="10"/>
@@ -6461,7 +6490,7 @@
       <c r="N249" s="10"/>
       <c r="O249" s="10"/>
     </row>
-    <row r="250" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A250" s="10"/>
       <c r="B250" s="10"/>
       <c r="C250" s="10"/>
@@ -6481,7 +6510,7 @@
       <c r="N250" s="10"/>
       <c r="O250" s="10"/>
     </row>
-    <row r="251" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A251" s="10"/>
       <c r="B251" s="10"/>
       <c r="C251" s="10"/>
@@ -6501,7 +6530,7 @@
       <c r="N251" s="10"/>
       <c r="O251" s="10"/>
     </row>
-    <row r="252" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A252" s="10"/>
       <c r="B252" s="10"/>
       <c r="C252" s="10"/>
@@ -6521,7 +6550,7 @@
       <c r="N252" s="10"/>
       <c r="O252" s="10"/>
     </row>
-    <row r="253" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A253" s="10"/>
       <c r="B253" s="10"/>
       <c r="C253" s="10"/>
@@ -6541,7 +6570,7 @@
       <c r="N253" s="10"/>
       <c r="O253" s="10"/>
     </row>
-    <row r="254" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A254" s="10"/>
       <c r="B254" s="10"/>
       <c r="C254" s="10"/>
@@ -6561,7 +6590,7 @@
       <c r="N254" s="10"/>
       <c r="O254" s="10"/>
     </row>
-    <row r="255" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A255" s="10"/>
       <c r="B255" s="10"/>
       <c r="C255" s="10"/>
@@ -6581,7 +6610,7 @@
       <c r="N255" s="10"/>
       <c r="O255" s="10"/>
     </row>
-    <row r="256" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A256" s="10"/>
       <c r="B256" s="10"/>
       <c r="C256" s="10"/>
@@ -6601,7 +6630,7 @@
       <c r="N256" s="10"/>
       <c r="O256" s="10"/>
     </row>
-    <row r="257" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A257" s="10"/>
       <c r="B257" s="10"/>
       <c r="C257" s="10"/>
@@ -6621,7 +6650,7 @@
       <c r="N257" s="10"/>
       <c r="O257" s="10"/>
     </row>
-    <row r="258" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A258" s="10"/>
       <c r="B258" s="10"/>
       <c r="C258" s="10"/>
@@ -6641,7 +6670,7 @@
       <c r="N258" s="10"/>
       <c r="O258" s="10"/>
     </row>
-    <row r="259" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A259" s="10"/>
       <c r="B259" s="10"/>
       <c r="C259" s="10"/>
@@ -6661,7 +6690,7 @@
       <c r="N259" s="10"/>
       <c r="O259" s="10"/>
     </row>
-    <row r="260" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A260" s="10"/>
       <c r="B260" s="10"/>
       <c r="C260" s="10"/>
@@ -6681,7 +6710,7 @@
       <c r="N260" s="10"/>
       <c r="O260" s="10"/>
     </row>
-    <row r="261" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A261" s="10"/>
       <c r="B261" s="10"/>
       <c r="C261" s="10"/>
@@ -6701,7 +6730,7 @@
       <c r="N261" s="10"/>
       <c r="O261" s="10"/>
     </row>
-    <row r="262" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A262" s="10"/>
       <c r="B262" s="10"/>
       <c r="C262" s="10"/>
@@ -6721,7 +6750,7 @@
       <c r="N262" s="10"/>
       <c r="O262" s="10"/>
     </row>
-    <row r="263" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A263" s="10"/>
       <c r="B263" s="10"/>
       <c r="C263" s="10"/>
@@ -6741,7 +6770,7 @@
       <c r="N263" s="10"/>
       <c r="O263" s="10"/>
     </row>
-    <row r="264" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A264" s="10"/>
       <c r="B264" s="10"/>
       <c r="C264" s="10"/>
@@ -6761,7 +6790,7 @@
       <c r="N264" s="10"/>
       <c r="O264" s="10"/>
     </row>
-    <row r="265" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A265" s="10"/>
       <c r="B265" s="10"/>
       <c r="C265" s="10"/>
@@ -6781,7 +6810,7 @@
       <c r="N265" s="10"/>
       <c r="O265" s="10"/>
     </row>
-    <row r="266" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A266" s="10"/>
       <c r="B266" s="10"/>
       <c r="C266" s="10"/>
@@ -6801,7 +6830,7 @@
       <c r="N266" s="10"/>
       <c r="O266" s="10"/>
     </row>
-    <row r="267" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A267" s="10"/>
       <c r="B267" s="10"/>
       <c r="C267" s="10"/>
@@ -6821,7 +6850,7 @@
       <c r="N267" s="10"/>
       <c r="O267" s="10"/>
     </row>
-    <row r="268" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A268" s="10"/>
       <c r="B268" s="10"/>
       <c r="C268" s="10"/>
@@ -6841,7 +6870,7 @@
       <c r="N268" s="10"/>
       <c r="O268" s="10"/>
     </row>
-    <row r="269" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A269" s="10"/>
       <c r="B269" s="10"/>
       <c r="C269" s="10"/>
@@ -6861,7 +6890,7 @@
       <c r="N269" s="10"/>
       <c r="O269" s="10"/>
     </row>
-    <row r="270" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A270" s="10"/>
       <c r="B270" s="10"/>
       <c r="C270" s="10"/>
@@ -6881,7 +6910,7 @@
       <c r="N270" s="10"/>
       <c r="O270" s="10"/>
     </row>
-    <row r="271" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A271" s="10"/>
       <c r="B271" s="10"/>
       <c r="C271" s="10"/>
@@ -6901,7 +6930,7 @@
       <c r="N271" s="10"/>
       <c r="O271" s="10"/>
     </row>
-    <row r="272" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A272" s="10"/>
       <c r="B272" s="10"/>
       <c r="C272" s="10"/>
@@ -6921,7 +6950,7 @@
       <c r="N272" s="10"/>
       <c r="O272" s="10"/>
     </row>
-    <row r="273" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A273" s="10"/>
       <c r="B273" s="10"/>
       <c r="C273" s="10"/>
@@ -6941,7 +6970,7 @@
       <c r="N273" s="10"/>
       <c r="O273" s="10"/>
     </row>
-    <row r="274" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A274" s="10"/>
       <c r="B274" s="10"/>
       <c r="C274" s="10"/>
@@ -6961,7 +6990,7 @@
       <c r="N274" s="10"/>
       <c r="O274" s="10"/>
     </row>
-    <row r="275" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A275" s="10"/>
       <c r="B275" s="10"/>
       <c r="C275" s="10"/>
@@ -6981,7 +7010,7 @@
       <c r="N275" s="10"/>
       <c r="O275" s="10"/>
     </row>
-    <row r="276" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A276" s="10"/>
       <c r="B276" s="10"/>
       <c r="C276" s="10"/>
@@ -7001,7 +7030,7 @@
       <c r="N276" s="10"/>
       <c r="O276" s="10"/>
     </row>
-    <row r="277" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A277" s="10"/>
       <c r="B277" s="10"/>
       <c r="C277" s="10"/>
@@ -7021,7 +7050,7 @@
       <c r="N277" s="10"/>
       <c r="O277" s="10"/>
     </row>
-    <row r="278" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A278" s="10"/>
       <c r="B278" s="10"/>
       <c r="C278" s="10"/>
@@ -7041,7 +7070,7 @@
       <c r="N278" s="10"/>
       <c r="O278" s="10"/>
     </row>
-    <row r="279" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A279" s="10"/>
       <c r="B279" s="10"/>
       <c r="C279" s="10"/>
@@ -7061,7 +7090,7 @@
       <c r="N279" s="10"/>
       <c r="O279" s="10"/>
     </row>
-    <row r="280" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A280" s="10"/>
       <c r="B280" s="10"/>
       <c r="C280" s="10"/>
@@ -7081,7 +7110,7 @@
       <c r="N280" s="10"/>
       <c r="O280" s="10"/>
     </row>
-    <row r="281" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A281" s="10"/>
       <c r="B281" s="10"/>
       <c r="C281" s="10"/>
@@ -7101,7 +7130,7 @@
       <c r="N281" s="10"/>
       <c r="O281" s="10"/>
     </row>
-    <row r="282" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A282" s="10"/>
       <c r="B282" s="10"/>
       <c r="C282" s="10"/>
@@ -7121,7 +7150,7 @@
       <c r="N282" s="10"/>
       <c r="O282" s="10"/>
     </row>
-    <row r="283" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A283" s="10"/>
       <c r="B283" s="10"/>
       <c r="C283" s="10"/>
@@ -7141,7 +7170,7 @@
       <c r="N283" s="10"/>
       <c r="O283" s="10"/>
     </row>
-    <row r="284" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A284" s="10"/>
       <c r="B284" s="10"/>
       <c r="C284" s="10"/>
@@ -7161,7 +7190,7 @@
       <c r="N284" s="10"/>
       <c r="O284" s="10"/>
     </row>
-    <row r="285" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A285" s="10"/>
       <c r="B285" s="10"/>
       <c r="C285" s="10"/>
@@ -7181,7 +7210,7 @@
       <c r="N285" s="10"/>
       <c r="O285" s="10"/>
     </row>
-    <row r="286" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A286" s="10"/>
       <c r="B286" s="10"/>
       <c r="C286" s="10"/>
@@ -7201,7 +7230,7 @@
       <c r="N286" s="10"/>
       <c r="O286" s="10"/>
     </row>
-    <row r="287" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A287" s="10"/>
       <c r="B287" s="10"/>
       <c r="C287" s="10"/>
@@ -7221,7 +7250,7 @@
       <c r="N287" s="10"/>
       <c r="O287" s="10"/>
     </row>
-    <row r="288" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A288" s="10"/>
       <c r="B288" s="10"/>
       <c r="C288" s="10"/>
@@ -7241,7 +7270,7 @@
       <c r="N288" s="10"/>
       <c r="O288" s="10"/>
     </row>
-    <row r="289" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A289" s="10"/>
       <c r="B289" s="10"/>
       <c r="C289" s="10"/>
@@ -7261,7 +7290,7 @@
       <c r="N289" s="10"/>
       <c r="O289" s="10"/>
     </row>
-    <row r="290" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A290" s="10"/>
       <c r="B290" s="10"/>
       <c r="C290" s="10"/>
@@ -7281,7 +7310,7 @@
       <c r="N290" s="10"/>
       <c r="O290" s="10"/>
     </row>
-    <row r="291" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A291" s="10"/>
       <c r="B291" s="10"/>
       <c r="C291" s="10"/>
@@ -7301,7 +7330,7 @@
       <c r="N291" s="10"/>
       <c r="O291" s="10"/>
     </row>
-    <row r="292" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A292" s="10"/>
       <c r="B292" s="10"/>
       <c r="C292" s="10"/>
@@ -7321,7 +7350,7 @@
       <c r="N292" s="10"/>
       <c r="O292" s="10"/>
     </row>
-    <row r="293" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A293" s="10"/>
       <c r="B293" s="10"/>
       <c r="C293" s="10"/>
@@ -7341,7 +7370,7 @@
       <c r="N293" s="10"/>
       <c r="O293" s="10"/>
     </row>
-    <row r="294" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A294" s="10"/>
       <c r="B294" s="10"/>
       <c r="C294" s="10"/>
@@ -7361,7 +7390,7 @@
       <c r="N294" s="10"/>
       <c r="O294" s="10"/>
     </row>
-    <row r="295" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A295" s="10"/>
       <c r="B295" s="10"/>
       <c r="C295" s="10"/>
@@ -7381,7 +7410,7 @@
       <c r="N295" s="10"/>
       <c r="O295" s="10"/>
     </row>
-    <row r="296" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A296" s="10"/>
       <c r="B296" s="10"/>
       <c r="C296" s="10"/>
@@ -7401,7 +7430,7 @@
       <c r="N296" s="10"/>
       <c r="O296" s="10"/>
     </row>
-    <row r="297" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A297" s="10"/>
       <c r="B297" s="10"/>
       <c r="C297" s="10"/>
@@ -7421,7 +7450,7 @@
       <c r="N297" s="10"/>
       <c r="O297" s="10"/>
     </row>
-    <row r="298" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A298" s="10"/>
       <c r="B298" s="10"/>
       <c r="C298" s="10"/>
@@ -7441,7 +7470,7 @@
       <c r="N298" s="10"/>
       <c r="O298" s="10"/>
     </row>
-    <row r="299" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A299" s="10"/>
       <c r="B299" s="10"/>
       <c r="C299" s="10"/>
@@ -7461,7 +7490,7 @@
       <c r="N299" s="10"/>
       <c r="O299" s="10"/>
     </row>
-    <row r="300" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A300" s="10"/>
       <c r="B300" s="10"/>
       <c r="C300" s="10"/>
@@ -7481,7 +7510,7 @@
       <c r="N300" s="10"/>
       <c r="O300" s="10"/>
     </row>
-    <row r="301" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A301" s="10"/>
       <c r="B301" s="10"/>
       <c r="C301" s="10"/>
@@ -7501,7 +7530,7 @@
       <c r="N301" s="10"/>
       <c r="O301" s="10"/>
     </row>
-    <row r="302" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A302" s="10"/>
       <c r="B302" s="10"/>
       <c r="C302" s="10"/>
@@ -7521,7 +7550,7 @@
       <c r="N302" s="10"/>
       <c r="O302" s="10"/>
     </row>
-    <row r="303" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A303" s="10"/>
       <c r="B303" s="10"/>
       <c r="C303" s="10"/>
@@ -7541,7 +7570,7 @@
       <c r="N303" s="10"/>
       <c r="O303" s="10"/>
     </row>
-    <row r="304" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A304" s="10"/>
       <c r="B304" s="10"/>
       <c r="C304" s="10"/>
@@ -7598,7 +7627,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -7606,7 +7635,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -7614,139 +7643,139 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D4" s="9"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="12">
         <v>10</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D5" s="12"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" s="12">
         <v>10</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="12">
         <v>10</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D7" s="12"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="12">
         <v>20</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D8" s="12"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B9" s="12">
         <v>10</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B10" s="12">
         <v>10</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D10" s="12"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B11" s="12">
         <v>10</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D11" s="12"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B12" s="12">
         <v>5</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D12" s="12"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B13" s="12">
         <v>5</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D13" s="12"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B14" s="12">
         <v>10</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D14" s="12"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B15" s="13">
         <f>SUM(B5:B14)</f>
@@ -7755,7 +7784,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -7789,7 +7818,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7803,7 +7832,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7817,34 +7846,34 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>11</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -13296,7 +13325,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -13305,7 +13334,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -13314,7 +13343,7 @@
     </row>
     <row r="3" ht="28.05" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B3"/>
       <c r="C3"/>
@@ -13323,41 +13352,41 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="7:11" x14ac:dyDescent="0.25">
       <c r="G4" s="17" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H4"/>
       <c r="J4" s="17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K4"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -13367,13 +13396,13 @@
       <c r="D6" s="22"/>
       <c r="E6" s="20"/>
       <c r="G6" s="23" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="K6" s="26">
         <f>SUMIF($A$6:$A$305,"panel",$C$6:$C$305)</f>
@@ -13387,13 +13416,13 @@
       <c r="D7" s="22"/>
       <c r="E7" s="20"/>
       <c r="G7" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J7" s="29" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K7" s="30">
         <f>SUMIF($A$6:$A$305,"inverter",$C$6:$C$305)</f>
@@ -13407,13 +13436,13 @@
       <c r="D8" s="22"/>
       <c r="E8" s="20"/>
       <c r="G8" s="23" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="J8" s="25" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K8" s="26">
         <f>SUMIF($A$6:$A$305,"mekanik",$C$6:$C$305)</f>
@@ -13427,13 +13456,13 @@
       <c r="D9" s="22"/>
       <c r="E9" s="20"/>
       <c r="G9" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K9" s="30">
         <f>SUMIF($A$6:$A$305,"elektrik_dc",$C$6:$C$305)</f>
@@ -13447,13 +13476,13 @@
       <c r="D10" s="22"/>
       <c r="E10" s="20"/>
       <c r="G10" s="23" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J10" s="25" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K10" s="26">
         <f>SUMIF($A$6:$A$305,"elektrik_ac",$C$6:$C$305)</f>
@@ -13467,13 +13496,13 @@
       <c r="D11" s="22"/>
       <c r="E11" s="20"/>
       <c r="G11" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H11" s="28" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J11" s="29" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K11" s="30">
         <f>SUMIF($A$6:$A$305,"elektrik_og",$C$6:$C$305)</f>
@@ -13487,13 +13516,13 @@
       <c r="D12" s="22"/>
       <c r="E12" s="20"/>
       <c r="G12" s="23" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H12" s="24" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J12" s="25" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K12" s="26">
         <f>SUMIF($A$6:$A$305,"enh",$C$6:$C$305)</f>
@@ -13507,13 +13536,13 @@
       <c r="D13" s="22"/>
       <c r="E13" s="20"/>
       <c r="G13" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H13" s="28" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J13" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K13" s="30">
         <f>SUMIF($A$6:$A$305,"altyapi",$C$6:$C$305)</f>
@@ -13527,13 +13556,13 @@
       <c r="D14" s="22"/>
       <c r="E14" s="20"/>
       <c r="G14" s="23" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H14" s="24" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="J14" s="25" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K14" s="26">
         <f>SUMIF($A$6:$A$305,"iscilik",$C$6:$C$305)</f>
@@ -13547,13 +13576,13 @@
       <c r="D15" s="22"/>
       <c r="E15" s="20"/>
       <c r="G15" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H15" s="28" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J15" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K15" s="30">
         <f>SUMIF($A$6:$A$305,"izin",$C$6:$C$305)</f>
@@ -13567,13 +13596,13 @@
       <c r="D16" s="22"/>
       <c r="E16" s="20"/>
       <c r="G16" s="23" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H16" s="24" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J16" s="25" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K16" s="26">
         <f>SUMIF($A$6:$A$305,"denetim",$C$6:$C$305)</f>
@@ -13587,13 +13616,13 @@
       <c r="D17" s="22"/>
       <c r="E17" s="20"/>
       <c r="G17" s="27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H17" s="28" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="J17" s="29" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K17" s="30">
         <f>SUMIF($A$6:$A$305,"diger",$C$6:$C$305)</f>
@@ -13607,7 +13636,7 @@
       <c r="D18" s="22"/>
       <c r="E18" s="20"/>
       <c r="J18" s="31" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K18" s="32">
         <f>SUM(K6:K17)</f>
@@ -13628,7 +13657,7 @@
       <c r="D20" s="22"/>
       <c r="E20" s="20"/>
       <c r="J20" s="33" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="K20" s="34">
         <f>COUNTIF($A$6:$A$305,"&lt;&gt;")</f>
@@ -15677,7 +15706,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -15692,7 +15721,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -15707,37 +15736,37 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -19666,7 +19695,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -19676,120 +19705,122 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
       <c r="D1"/>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
       <c r="D2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>132</v>
+        <v>134</v>
+      </c>
+      <c r="E5" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="6" ht="57" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="7" ht="28.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" ht="28.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>138</v>
+        <v>141</v>
+      </c>
+      <c r="E7" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="11" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="3:3" x14ac:dyDescent="0.25"/>
+        <v>151</v>
+      </c>
+    </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C13" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C14" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C15" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(proje-ekleme): sihirbaz ve Excel ile proje ekleme (proje kodu, PM yetkisi, Excel v8)
- Sihirbaz: Proje Kodu alanı (faz-a ile aynı); yeni proje create_project_with_code ile (proje + kod tek işlemde, PM de açabilir)
- Tedarik onayı yeni projede isteğe bağlı; tedarik RPC'si yalnızca onay verildiyse çağrılır (Karar 88)
- Excel şablonu v8 (E13 proje kodu, faz-a ile aynı dosya); export E13'ü yazar
- import-project-excel: yeni proje create_project_with_code ile; güncellemede E13 kontrolü (Karar 57/60) ve rol kontrolü (admin/PM);
  risk varsayılanları Türkçe (açık/yüksek/düşük); yazmadan önce bütün satırlar doğrulanır; kopya kodu E13'ten
- Varsayılan kategori ağırlıkları 15 kategori (Karar 89; DB trigger ayrıca uygulanacak)
- supabase/migrations/20261014102306_f1_a1_a3_proje_olusturma.sql: canlıya uygulanan F1 A1-A3

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/excel/fons-solar-proje-sablonu.xlsx
+++ b/public/excel/fons-solar-proje-sablonu.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="160">
   <si>
     <t xml:space="preserve">  FONS SOLAR   |   PROJE BİLGİLERİ</t>
   </si>
@@ -74,6 +74,12 @@
   </si>
   <si>
     <t>← Başlangıç ve bitiş tarihlerinden otomatik</t>
+  </si>
+  <si>
+    <t>Proje Kodu *</t>
+  </si>
+  <si>
+    <t>2-5 karakter, harfle başlar, büyük harf/rakam (ör. DYB). Sonradan değiştirilemez</t>
   </si>
   <si>
     <t>GÜÇ BİLGİLERİ</t>
@@ -428,7 +434,7 @@
     <t xml:space="preserve">  FONS SOLAR   |   KULLANIM KILAVUZU</t>
   </si>
   <si>
-    <t>Şablon v7 (03.08.2026: İş Kalemleri'nden Dashboard Göster/Sıra ve Kritik mi? kolonları kaldırıldı)</t>
+    <t>Şablon v8 (12.10.2026: Proje Bilgileri E13 Proje Kodu eklendi; ağırlıksız kategoriye görev yazılamaz)</t>
   </si>
   <si>
     <t>1️⃣</t>
@@ -438,6 +444,9 @@
   </si>
   <si>
     <t>Proje ID: küçük harf, boşluksuz, tire. Tür ve Durum dropdown. Toplam Gün otomatik.</t>
+  </si>
+  <si>
+    <t>Proje ID: küçük harf, boşluksuz, tire. Proje Kodu (E13): 2-5 karakter, harfle başlar, büyük harf/rakam (ör. DYB); yeni projede zorunlu, sonradan değiştirilemez. Mevcut projeyi güncellerken E13 projenin koduyla aynı olmalı, yoksa yükleme reddedilir. Tür ve Durum dropdown. Toplam Gün otomatik.</t>
   </si>
   <si>
     <t>2️⃣</t>
@@ -456,6 +465,9 @@
   </si>
   <si>
     <t>Genel proje ilerlemesi bu 10 sabit kategorinin ağırlıklı ortalamasıdır. Buradan veri içeri aktarılmaz — görevleri doğru Kategori'ye atamak yeterlidir.</t>
+  </si>
+  <si>
+    <t>Genel proje ilerlemesi ağırlık tablosundaki kategorilerin ağırlıklı ortalamasıdır. Buradan veri içeri aktarılmaz. Ağırlık tablosunda olmayan kategoriye görev yazılamaz: önce ağırlık tanımlayın, fiziksel değilse %0 girin.</t>
   </si>
   <si>
     <t>4️⃣</t>
@@ -1277,9 +1289,21 @@
         <v>17</v>
       </c>
     </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13" s="5"/>
+      <c r="F13"/>
+      <c r="H13" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B14"/>
       <c r="C14"/>
@@ -1295,43 +1319,43 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C15"/>
       <c r="D15"/>
       <c r="E15" s="5"/>
       <c r="F15" s="6"/>
       <c r="H15" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16" s="5"/>
       <c r="F16" s="6"/>
       <c r="H16" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C17"/>
       <c r="D17"/>
       <c r="E17" s="5"/>
       <c r="F17" s="6"/>
       <c r="H17" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1347,52 +1371,52 @@
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C20"/>
       <c r="D20"/>
       <c r="E20" s="5"/>
       <c r="F20" s="6"/>
       <c r="H20" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J20" s="5"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C21"/>
       <c r="D21"/>
       <c r="E21" s="5"/>
       <c r="F21" s="6"/>
       <c r="H21" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J21" s="5"/>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C22"/>
       <c r="D22"/>
       <c r="E22" s="5"/>
       <c r="F22" s="6"/>
       <c r="H22" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="J22" s="5"/>
     </row>
     <row r="23" spans="8:10" x14ac:dyDescent="0.25">
       <c r="H23" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J23" s="5"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B25"/>
       <c r="C25"/>
@@ -1407,7 +1431,7 @@
       <c r="L25"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="36">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A4:L4"/>
@@ -1427,6 +1451,8 @@
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:F13"/>
     <mergeCell ref="A14:L14"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="E15:F15"/>
@@ -1443,7 +1469,10 @@
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="A25:L25"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Proje kodu" error="2-5 karakter, harfle başlar, yalnızca büyük harf ve rakam (ör. DYB, ADN1)." sqref="E13">
+      <formula1>AND(LEN(E13)&gt;=2,LEN(E13)&lt;=5,EXACT(E13,UPPER(E13)),ISERROR(VALUE(LEFT(E13,1))))</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="E8">
       <formula1>"Arazi GES,Endüstriyel Çatı GES,Evsel GES"</formula1>
     </dataValidation>
@@ -1514,54 +1543,54 @@
       <c r="Q2"/>
       <c r="R2"/>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>11</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N4" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -1581,7 +1610,7 @@
       <c r="N5" s="10"/>
       <c r="O5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -1601,7 +1630,7 @@
       <c r="N6" s="10"/>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -1621,7 +1650,7 @@
       <c r="N7" s="10"/>
       <c r="O7" s="10"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -1641,7 +1670,7 @@
       <c r="N8" s="10"/>
       <c r="O8" s="10"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -1661,7 +1690,7 @@
       <c r="N9" s="10"/>
       <c r="O9" s="10"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -1681,7 +1710,7 @@
       <c r="N10" s="10"/>
       <c r="O10" s="10"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -1701,7 +1730,7 @@
       <c r="N11" s="10"/>
       <c r="O11" s="10"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -1721,7 +1750,7 @@
       <c r="N12" s="10"/>
       <c r="O12" s="10"/>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1741,7 +1770,7 @@
       <c r="N13" s="10"/>
       <c r="O13" s="10"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -1761,7 +1790,7 @@
       <c r="N14" s="10"/>
       <c r="O14" s="10"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -1781,7 +1810,7 @@
       <c r="N15" s="10"/>
       <c r="O15" s="10"/>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -1801,7 +1830,7 @@
       <c r="N16" s="10"/>
       <c r="O16" s="10"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -1821,7 +1850,7 @@
       <c r="N17" s="10"/>
       <c r="O17" s="10"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -1841,7 +1870,7 @@
       <c r="N18" s="10"/>
       <c r="O18" s="10"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="10"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
@@ -1861,7 +1890,7 @@
       <c r="N19" s="10"/>
       <c r="O19" s="10"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -1881,7 +1910,7 @@
       <c r="N20" s="10"/>
       <c r="O20" s="10"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -1901,7 +1930,7 @@
       <c r="N21" s="10"/>
       <c r="O21" s="10"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -1921,7 +1950,7 @@
       <c r="N22" s="10"/>
       <c r="O22" s="10"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
@@ -1941,7 +1970,7 @@
       <c r="N23" s="10"/>
       <c r="O23" s="10"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -1961,7 +1990,7 @@
       <c r="N24" s="10"/>
       <c r="O24" s="10"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -1981,7 +2010,7 @@
       <c r="N25" s="10"/>
       <c r="O25" s="10"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -2001,7 +2030,7 @@
       <c r="N26" s="10"/>
       <c r="O26" s="10"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -2021,7 +2050,7 @@
       <c r="N27" s="10"/>
       <c r="O27" s="10"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -2041,7 +2070,7 @@
       <c r="N28" s="10"/>
       <c r="O28" s="10"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -2061,7 +2090,7 @@
       <c r="N29" s="10"/>
       <c r="O29" s="10"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -2081,7 +2110,7 @@
       <c r="N30" s="10"/>
       <c r="O30" s="10"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
@@ -2101,7 +2130,7 @@
       <c r="N31" s="10"/>
       <c r="O31" s="10"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
@@ -2121,7 +2150,7 @@
       <c r="N32" s="10"/>
       <c r="O32" s="10"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
@@ -2141,7 +2170,7 @@
       <c r="N33" s="10"/>
       <c r="O33" s="10"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -2161,7 +2190,7 @@
       <c r="N34" s="10"/>
       <c r="O34" s="10"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -2181,7 +2210,7 @@
       <c r="N35" s="10"/>
       <c r="O35" s="10"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
@@ -2201,7 +2230,7 @@
       <c r="N36" s="10"/>
       <c r="O36" s="10"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -2221,7 +2250,7 @@
       <c r="N37" s="10"/>
       <c r="O37" s="10"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="10"/>
       <c r="B38" s="10"/>
       <c r="C38" s="10"/>
@@ -2241,7 +2270,7 @@
       <c r="N38" s="10"/>
       <c r="O38" s="10"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="10"/>
       <c r="B39" s="10"/>
       <c r="C39" s="10"/>
@@ -2261,7 +2290,7 @@
       <c r="N39" s="10"/>
       <c r="O39" s="10"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="10"/>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
@@ -2281,7 +2310,7 @@
       <c r="N40" s="10"/>
       <c r="O40" s="10"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
       <c r="B41" s="10"/>
       <c r="C41" s="10"/>
@@ -2301,7 +2330,7 @@
       <c r="N41" s="10"/>
       <c r="O41" s="10"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="10"/>
       <c r="B42" s="10"/>
       <c r="C42" s="10"/>
@@ -2321,7 +2350,7 @@
       <c r="N42" s="10"/>
       <c r="O42" s="10"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
@@ -2341,7 +2370,7 @@
       <c r="N43" s="10"/>
       <c r="O43" s="10"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="10"/>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
@@ -2361,7 +2390,7 @@
       <c r="N44" s="10"/>
       <c r="O44" s="10"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="10"/>
       <c r="B45" s="10"/>
       <c r="C45" s="10"/>
@@ -2381,7 +2410,7 @@
       <c r="N45" s="10"/>
       <c r="O45" s="10"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="10"/>
       <c r="B46" s="10"/>
       <c r="C46" s="10"/>
@@ -2401,7 +2430,7 @@
       <c r="N46" s="10"/>
       <c r="O46" s="10"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
       <c r="C47" s="10"/>
@@ -2421,7 +2450,7 @@
       <c r="N47" s="10"/>
       <c r="O47" s="10"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="10"/>
       <c r="B48" s="10"/>
       <c r="C48" s="10"/>
@@ -2441,7 +2470,7 @@
       <c r="N48" s="10"/>
       <c r="O48" s="10"/>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="10"/>
       <c r="B49" s="10"/>
       <c r="C49" s="10"/>
@@ -2461,7 +2490,7 @@
       <c r="N49" s="10"/>
       <c r="O49" s="10"/>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A50" s="10"/>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
@@ -2481,7 +2510,7 @@
       <c r="N50" s="10"/>
       <c r="O50" s="10"/>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="10"/>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
@@ -2501,7 +2530,7 @@
       <c r="N51" s="10"/>
       <c r="O51" s="10"/>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="10"/>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
@@ -2521,7 +2550,7 @@
       <c r="N52" s="10"/>
       <c r="O52" s="10"/>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="10"/>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
@@ -2541,7 +2570,7 @@
       <c r="N53" s="10"/>
       <c r="O53" s="10"/>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="10"/>
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
@@ -2561,7 +2590,7 @@
       <c r="N54" s="10"/>
       <c r="O54" s="10"/>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="10"/>
       <c r="B55" s="10"/>
       <c r="C55" s="10"/>
@@ -2581,7 +2610,7 @@
       <c r="N55" s="10"/>
       <c r="O55" s="10"/>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="10"/>
       <c r="B56" s="10"/>
       <c r="C56" s="10"/>
@@ -2601,7 +2630,7 @@
       <c r="N56" s="10"/>
       <c r="O56" s="10"/>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="10"/>
       <c r="B57" s="10"/>
       <c r="C57" s="10"/>
@@ -2621,7 +2650,7 @@
       <c r="N57" s="10"/>
       <c r="O57" s="10"/>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="10"/>
       <c r="B58" s="10"/>
       <c r="C58" s="10"/>
@@ -2641,7 +2670,7 @@
       <c r="N58" s="10"/>
       <c r="O58" s="10"/>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="10"/>
       <c r="B59" s="10"/>
       <c r="C59" s="10"/>
@@ -2661,7 +2690,7 @@
       <c r="N59" s="10"/>
       <c r="O59" s="10"/>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="10"/>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
@@ -2681,7 +2710,7 @@
       <c r="N60" s="10"/>
       <c r="O60" s="10"/>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="10"/>
       <c r="B61" s="10"/>
       <c r="C61" s="10"/>
@@ -2701,7 +2730,7 @@
       <c r="N61" s="10"/>
       <c r="O61" s="10"/>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="10"/>
       <c r="B62" s="10"/>
       <c r="C62" s="10"/>
@@ -2721,7 +2750,7 @@
       <c r="N62" s="10"/>
       <c r="O62" s="10"/>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="10"/>
       <c r="B63" s="10"/>
       <c r="C63" s="10"/>
@@ -2741,7 +2770,7 @@
       <c r="N63" s="10"/>
       <c r="O63" s="10"/>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="10"/>
       <c r="B64" s="10"/>
       <c r="C64" s="10"/>
@@ -2761,7 +2790,7 @@
       <c r="N64" s="10"/>
       <c r="O64" s="10"/>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="10"/>
       <c r="B65" s="10"/>
       <c r="C65" s="10"/>
@@ -2781,7 +2810,7 @@
       <c r="N65" s="10"/>
       <c r="O65" s="10"/>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="10"/>
       <c r="B66" s="10"/>
       <c r="C66" s="10"/>
@@ -2801,7 +2830,7 @@
       <c r="N66" s="10"/>
       <c r="O66" s="10"/>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="10"/>
       <c r="B67" s="10"/>
       <c r="C67" s="10"/>
@@ -2821,7 +2850,7 @@
       <c r="N67" s="10"/>
       <c r="O67" s="10"/>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="10"/>
       <c r="B68" s="10"/>
       <c r="C68" s="10"/>
@@ -2841,7 +2870,7 @@
       <c r="N68" s="10"/>
       <c r="O68" s="10"/>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="10"/>
       <c r="B69" s="10"/>
       <c r="C69" s="10"/>
@@ -2861,7 +2890,7 @@
       <c r="N69" s="10"/>
       <c r="O69" s="10"/>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="10"/>
       <c r="B70" s="10"/>
       <c r="C70" s="10"/>
@@ -2881,7 +2910,7 @@
       <c r="N70" s="10"/>
       <c r="O70" s="10"/>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="10"/>
       <c r="B71" s="10"/>
       <c r="C71" s="10"/>
@@ -2901,7 +2930,7 @@
       <c r="N71" s="10"/>
       <c r="O71" s="10"/>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="10"/>
       <c r="B72" s="10"/>
       <c r="C72" s="10"/>
@@ -2921,7 +2950,7 @@
       <c r="N72" s="10"/>
       <c r="O72" s="10"/>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="10"/>
       <c r="B73" s="10"/>
       <c r="C73" s="10"/>
@@ -2941,7 +2970,7 @@
       <c r="N73" s="10"/>
       <c r="O73" s="10"/>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="10"/>
       <c r="B74" s="10"/>
       <c r="C74" s="10"/>
@@ -2961,7 +2990,7 @@
       <c r="N74" s="10"/>
       <c r="O74" s="10"/>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="10"/>
       <c r="B75" s="10"/>
       <c r="C75" s="10"/>
@@ -2981,7 +3010,7 @@
       <c r="N75" s="10"/>
       <c r="O75" s="10"/>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" s="10"/>
       <c r="B76" s="10"/>
       <c r="C76" s="10"/>
@@ -3001,7 +3030,7 @@
       <c r="N76" s="10"/>
       <c r="O76" s="10"/>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" s="10"/>
       <c r="B77" s="10"/>
       <c r="C77" s="10"/>
@@ -3021,7 +3050,7 @@
       <c r="N77" s="10"/>
       <c r="O77" s="10"/>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A78" s="10"/>
       <c r="B78" s="10"/>
       <c r="C78" s="10"/>
@@ -3041,7 +3070,7 @@
       <c r="N78" s="10"/>
       <c r="O78" s="10"/>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="10"/>
       <c r="B79" s="10"/>
       <c r="C79" s="10"/>
@@ -3061,7 +3090,7 @@
       <c r="N79" s="10"/>
       <c r="O79" s="10"/>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" s="10"/>
       <c r="B80" s="10"/>
       <c r="C80" s="10"/>
@@ -3081,7 +3110,7 @@
       <c r="N80" s="10"/>
       <c r="O80" s="10"/>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A81" s="10"/>
       <c r="B81" s="10"/>
       <c r="C81" s="10"/>
@@ -3101,7 +3130,7 @@
       <c r="N81" s="10"/>
       <c r="O81" s="10"/>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A82" s="10"/>
       <c r="B82" s="10"/>
       <c r="C82" s="10"/>
@@ -3121,7 +3150,7 @@
       <c r="N82" s="10"/>
       <c r="O82" s="10"/>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A83" s="10"/>
       <c r="B83" s="10"/>
       <c r="C83" s="10"/>
@@ -3141,7 +3170,7 @@
       <c r="N83" s="10"/>
       <c r="O83" s="10"/>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A84" s="10"/>
       <c r="B84" s="10"/>
       <c r="C84" s="10"/>
@@ -3161,7 +3190,7 @@
       <c r="N84" s="10"/>
       <c r="O84" s="10"/>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A85" s="10"/>
       <c r="B85" s="10"/>
       <c r="C85" s="10"/>
@@ -3181,7 +3210,7 @@
       <c r="N85" s="10"/>
       <c r="O85" s="10"/>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A86" s="10"/>
       <c r="B86" s="10"/>
       <c r="C86" s="10"/>
@@ -3201,7 +3230,7 @@
       <c r="N86" s="10"/>
       <c r="O86" s="10"/>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A87" s="10"/>
       <c r="B87" s="10"/>
       <c r="C87" s="10"/>
@@ -3221,7 +3250,7 @@
       <c r="N87" s="10"/>
       <c r="O87" s="10"/>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A88" s="10"/>
       <c r="B88" s="10"/>
       <c r="C88" s="10"/>
@@ -3241,7 +3270,7 @@
       <c r="N88" s="10"/>
       <c r="O88" s="10"/>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A89" s="10"/>
       <c r="B89" s="10"/>
       <c r="C89" s="10"/>
@@ -3261,7 +3290,7 @@
       <c r="N89" s="10"/>
       <c r="O89" s="10"/>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A90" s="10"/>
       <c r="B90" s="10"/>
       <c r="C90" s="10"/>
@@ -3281,7 +3310,7 @@
       <c r="N90" s="10"/>
       <c r="O90" s="10"/>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A91" s="10"/>
       <c r="B91" s="10"/>
       <c r="C91" s="10"/>
@@ -3301,7 +3330,7 @@
       <c r="N91" s="10"/>
       <c r="O91" s="10"/>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A92" s="10"/>
       <c r="B92" s="10"/>
       <c r="C92" s="10"/>
@@ -3321,7 +3350,7 @@
       <c r="N92" s="10"/>
       <c r="O92" s="10"/>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A93" s="10"/>
       <c r="B93" s="10"/>
       <c r="C93" s="10"/>
@@ -3341,7 +3370,7 @@
       <c r="N93" s="10"/>
       <c r="O93" s="10"/>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A94" s="10"/>
       <c r="B94" s="10"/>
       <c r="C94" s="10"/>
@@ -3361,7 +3390,7 @@
       <c r="N94" s="10"/>
       <c r="O94" s="10"/>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A95" s="10"/>
       <c r="B95" s="10"/>
       <c r="C95" s="10"/>
@@ -3381,7 +3410,7 @@
       <c r="N95" s="10"/>
       <c r="O95" s="10"/>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A96" s="10"/>
       <c r="B96" s="10"/>
       <c r="C96" s="10"/>
@@ -3401,7 +3430,7 @@
       <c r="N96" s="10"/>
       <c r="O96" s="10"/>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A97" s="10"/>
       <c r="B97" s="10"/>
       <c r="C97" s="10"/>
@@ -3421,7 +3450,7 @@
       <c r="N97" s="10"/>
       <c r="O97" s="10"/>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A98" s="10"/>
       <c r="B98" s="10"/>
       <c r="C98" s="10"/>
@@ -3441,7 +3470,7 @@
       <c r="N98" s="10"/>
       <c r="O98" s="10"/>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A99" s="10"/>
       <c r="B99" s="10"/>
       <c r="C99" s="10"/>
@@ -3461,7 +3490,7 @@
       <c r="N99" s="10"/>
       <c r="O99" s="10"/>
     </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A100" s="10"/>
       <c r="B100" s="10"/>
       <c r="C100" s="10"/>
@@ -3481,7 +3510,7 @@
       <c r="N100" s="10"/>
       <c r="O100" s="10"/>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A101" s="10"/>
       <c r="B101" s="10"/>
       <c r="C101" s="10"/>
@@ -3501,7 +3530,7 @@
       <c r="N101" s="10"/>
       <c r="O101" s="10"/>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A102" s="10"/>
       <c r="B102" s="10"/>
       <c r="C102" s="10"/>
@@ -3521,7 +3550,7 @@
       <c r="N102" s="10"/>
       <c r="O102" s="10"/>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A103" s="10"/>
       <c r="B103" s="10"/>
       <c r="C103" s="10"/>
@@ -3541,7 +3570,7 @@
       <c r="N103" s="10"/>
       <c r="O103" s="10"/>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A104" s="10"/>
       <c r="B104" s="10"/>
       <c r="C104" s="10"/>
@@ -3561,7 +3590,7 @@
       <c r="N104" s="10"/>
       <c r="O104" s="10"/>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A105" s="10"/>
       <c r="B105" s="10"/>
       <c r="C105" s="10"/>
@@ -3581,7 +3610,7 @@
       <c r="N105" s="10"/>
       <c r="O105" s="10"/>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A106" s="10"/>
       <c r="B106" s="10"/>
       <c r="C106" s="10"/>
@@ -3601,7 +3630,7 @@
       <c r="N106" s="10"/>
       <c r="O106" s="10"/>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A107" s="10"/>
       <c r="B107" s="10"/>
       <c r="C107" s="10"/>
@@ -3621,7 +3650,7 @@
       <c r="N107" s="10"/>
       <c r="O107" s="10"/>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A108" s="10"/>
       <c r="B108" s="10"/>
       <c r="C108" s="10"/>
@@ -3641,7 +3670,7 @@
       <c r="N108" s="10"/>
       <c r="O108" s="10"/>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A109" s="10"/>
       <c r="B109" s="10"/>
       <c r="C109" s="10"/>
@@ -3661,7 +3690,7 @@
       <c r="N109" s="10"/>
       <c r="O109" s="10"/>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A110" s="10"/>
       <c r="B110" s="10"/>
       <c r="C110" s="10"/>
@@ -3681,7 +3710,7 @@
       <c r="N110" s="10"/>
       <c r="O110" s="10"/>
     </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A111" s="10"/>
       <c r="B111" s="10"/>
       <c r="C111" s="10"/>
@@ -3701,7 +3730,7 @@
       <c r="N111" s="10"/>
       <c r="O111" s="10"/>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A112" s="10"/>
       <c r="B112" s="10"/>
       <c r="C112" s="10"/>
@@ -3721,7 +3750,7 @@
       <c r="N112" s="10"/>
       <c r="O112" s="10"/>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A113" s="10"/>
       <c r="B113" s="10"/>
       <c r="C113" s="10"/>
@@ -3741,7 +3770,7 @@
       <c r="N113" s="10"/>
       <c r="O113" s="10"/>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A114" s="10"/>
       <c r="B114" s="10"/>
       <c r="C114" s="10"/>
@@ -3761,7 +3790,7 @@
       <c r="N114" s="10"/>
       <c r="O114" s="10"/>
     </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A115" s="10"/>
       <c r="B115" s="10"/>
       <c r="C115" s="10"/>
@@ -3781,7 +3810,7 @@
       <c r="N115" s="10"/>
       <c r="O115" s="10"/>
     </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A116" s="10"/>
       <c r="B116" s="10"/>
       <c r="C116" s="10"/>
@@ -3801,7 +3830,7 @@
       <c r="N116" s="10"/>
       <c r="O116" s="10"/>
     </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A117" s="10"/>
       <c r="B117" s="10"/>
       <c r="C117" s="10"/>
@@ -3821,7 +3850,7 @@
       <c r="N117" s="10"/>
       <c r="O117" s="10"/>
     </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A118" s="10"/>
       <c r="B118" s="10"/>
       <c r="C118" s="10"/>
@@ -3841,7 +3870,7 @@
       <c r="N118" s="10"/>
       <c r="O118" s="10"/>
     </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A119" s="10"/>
       <c r="B119" s="10"/>
       <c r="C119" s="10"/>
@@ -3861,7 +3890,7 @@
       <c r="N119" s="10"/>
       <c r="O119" s="10"/>
     </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A120" s="10"/>
       <c r="B120" s="10"/>
       <c r="C120" s="10"/>
@@ -3881,7 +3910,7 @@
       <c r="N120" s="10"/>
       <c r="O120" s="10"/>
     </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A121" s="10"/>
       <c r="B121" s="10"/>
       <c r="C121" s="10"/>
@@ -3901,7 +3930,7 @@
       <c r="N121" s="10"/>
       <c r="O121" s="10"/>
     </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A122" s="10"/>
       <c r="B122" s="10"/>
       <c r="C122" s="10"/>
@@ -3921,7 +3950,7 @@
       <c r="N122" s="10"/>
       <c r="O122" s="10"/>
     </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A123" s="10"/>
       <c r="B123" s="10"/>
       <c r="C123" s="10"/>
@@ -3941,7 +3970,7 @@
       <c r="N123" s="10"/>
       <c r="O123" s="10"/>
     </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A124" s="10"/>
       <c r="B124" s="10"/>
       <c r="C124" s="10"/>
@@ -3961,7 +3990,7 @@
       <c r="N124" s="10"/>
       <c r="O124" s="10"/>
     </row>
-    <row r="125" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A125" s="10"/>
       <c r="B125" s="10"/>
       <c r="C125" s="10"/>
@@ -3981,7 +4010,7 @@
       <c r="N125" s="10"/>
       <c r="O125" s="10"/>
     </row>
-    <row r="126" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A126" s="10"/>
       <c r="B126" s="10"/>
       <c r="C126" s="10"/>
@@ -4001,7 +4030,7 @@
       <c r="N126" s="10"/>
       <c r="O126" s="10"/>
     </row>
-    <row r="127" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A127" s="10"/>
       <c r="B127" s="10"/>
       <c r="C127" s="10"/>
@@ -4021,7 +4050,7 @@
       <c r="N127" s="10"/>
       <c r="O127" s="10"/>
     </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A128" s="10"/>
       <c r="B128" s="10"/>
       <c r="C128" s="10"/>
@@ -4041,7 +4070,7 @@
       <c r="N128" s="10"/>
       <c r="O128" s="10"/>
     </row>
-    <row r="129" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A129" s="10"/>
       <c r="B129" s="10"/>
       <c r="C129" s="10"/>
@@ -4061,7 +4090,7 @@
       <c r="N129" s="10"/>
       <c r="O129" s="10"/>
     </row>
-    <row r="130" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A130" s="10"/>
       <c r="B130" s="10"/>
       <c r="C130" s="10"/>
@@ -4081,7 +4110,7 @@
       <c r="N130" s="10"/>
       <c r="O130" s="10"/>
     </row>
-    <row r="131" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A131" s="10"/>
       <c r="B131" s="10"/>
       <c r="C131" s="10"/>
@@ -4101,7 +4130,7 @@
       <c r="N131" s="10"/>
       <c r="O131" s="10"/>
     </row>
-    <row r="132" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A132" s="10"/>
       <c r="B132" s="10"/>
       <c r="C132" s="10"/>
@@ -4121,7 +4150,7 @@
       <c r="N132" s="10"/>
       <c r="O132" s="10"/>
     </row>
-    <row r="133" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A133" s="10"/>
       <c r="B133" s="10"/>
       <c r="C133" s="10"/>
@@ -4141,7 +4170,7 @@
       <c r="N133" s="10"/>
       <c r="O133" s="10"/>
     </row>
-    <row r="134" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A134" s="10"/>
       <c r="B134" s="10"/>
       <c r="C134" s="10"/>
@@ -4161,7 +4190,7 @@
       <c r="N134" s="10"/>
       <c r="O134" s="10"/>
     </row>
-    <row r="135" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A135" s="10"/>
       <c r="B135" s="10"/>
       <c r="C135" s="10"/>
@@ -4181,7 +4210,7 @@
       <c r="N135" s="10"/>
       <c r="O135" s="10"/>
     </row>
-    <row r="136" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A136" s="10"/>
       <c r="B136" s="10"/>
       <c r="C136" s="10"/>
@@ -4201,7 +4230,7 @@
       <c r="N136" s="10"/>
       <c r="O136" s="10"/>
     </row>
-    <row r="137" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A137" s="10"/>
       <c r="B137" s="10"/>
       <c r="C137" s="10"/>
@@ -4221,7 +4250,7 @@
       <c r="N137" s="10"/>
       <c r="O137" s="10"/>
     </row>
-    <row r="138" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A138" s="10"/>
       <c r="B138" s="10"/>
       <c r="C138" s="10"/>
@@ -4241,7 +4270,7 @@
       <c r="N138" s="10"/>
       <c r="O138" s="10"/>
     </row>
-    <row r="139" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A139" s="10"/>
       <c r="B139" s="10"/>
       <c r="C139" s="10"/>
@@ -4261,7 +4290,7 @@
       <c r="N139" s="10"/>
       <c r="O139" s="10"/>
     </row>
-    <row r="140" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A140" s="10"/>
       <c r="B140" s="10"/>
       <c r="C140" s="10"/>
@@ -4281,7 +4310,7 @@
       <c r="N140" s="10"/>
       <c r="O140" s="10"/>
     </row>
-    <row r="141" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A141" s="10"/>
       <c r="B141" s="10"/>
       <c r="C141" s="10"/>
@@ -4301,7 +4330,7 @@
       <c r="N141" s="10"/>
       <c r="O141" s="10"/>
     </row>
-    <row r="142" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A142" s="10"/>
       <c r="B142" s="10"/>
       <c r="C142" s="10"/>
@@ -4321,7 +4350,7 @@
       <c r="N142" s="10"/>
       <c r="O142" s="10"/>
     </row>
-    <row r="143" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A143" s="10"/>
       <c r="B143" s="10"/>
       <c r="C143" s="10"/>
@@ -4341,7 +4370,7 @@
       <c r="N143" s="10"/>
       <c r="O143" s="10"/>
     </row>
-    <row r="144" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A144" s="10"/>
       <c r="B144" s="10"/>
       <c r="C144" s="10"/>
@@ -4361,7 +4390,7 @@
       <c r="N144" s="10"/>
       <c r="O144" s="10"/>
     </row>
-    <row r="145" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A145" s="10"/>
       <c r="B145" s="10"/>
       <c r="C145" s="10"/>
@@ -4381,7 +4410,7 @@
       <c r="N145" s="10"/>
       <c r="O145" s="10"/>
     </row>
-    <row r="146" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A146" s="10"/>
       <c r="B146" s="10"/>
       <c r="C146" s="10"/>
@@ -4401,7 +4430,7 @@
       <c r="N146" s="10"/>
       <c r="O146" s="10"/>
     </row>
-    <row r="147" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A147" s="10"/>
       <c r="B147" s="10"/>
       <c r="C147" s="10"/>
@@ -4421,7 +4450,7 @@
       <c r="N147" s="10"/>
       <c r="O147" s="10"/>
     </row>
-    <row r="148" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A148" s="10"/>
       <c r="B148" s="10"/>
       <c r="C148" s="10"/>
@@ -4441,7 +4470,7 @@
       <c r="N148" s="10"/>
       <c r="O148" s="10"/>
     </row>
-    <row r="149" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A149" s="10"/>
       <c r="B149" s="10"/>
       <c r="C149" s="10"/>
@@ -4461,7 +4490,7 @@
       <c r="N149" s="10"/>
       <c r="O149" s="10"/>
     </row>
-    <row r="150" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A150" s="10"/>
       <c r="B150" s="10"/>
       <c r="C150" s="10"/>
@@ -4481,7 +4510,7 @@
       <c r="N150" s="10"/>
       <c r="O150" s="10"/>
     </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A151" s="10"/>
       <c r="B151" s="10"/>
       <c r="C151" s="10"/>
@@ -4501,7 +4530,7 @@
       <c r="N151" s="10"/>
       <c r="O151" s="10"/>
     </row>
-    <row r="152" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A152" s="10"/>
       <c r="B152" s="10"/>
       <c r="C152" s="10"/>
@@ -4521,7 +4550,7 @@
       <c r="N152" s="10"/>
       <c r="O152" s="10"/>
     </row>
-    <row r="153" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A153" s="10"/>
       <c r="B153" s="10"/>
       <c r="C153" s="10"/>
@@ -4541,7 +4570,7 @@
       <c r="N153" s="10"/>
       <c r="O153" s="10"/>
     </row>
-    <row r="154" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A154" s="10"/>
       <c r="B154" s="10"/>
       <c r="C154" s="10"/>
@@ -4561,7 +4590,7 @@
       <c r="N154" s="10"/>
       <c r="O154" s="10"/>
     </row>
-    <row r="155" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A155" s="10"/>
       <c r="B155" s="10"/>
       <c r="C155" s="10"/>
@@ -4581,7 +4610,7 @@
       <c r="N155" s="10"/>
       <c r="O155" s="10"/>
     </row>
-    <row r="156" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A156" s="10"/>
       <c r="B156" s="10"/>
       <c r="C156" s="10"/>
@@ -4601,7 +4630,7 @@
       <c r="N156" s="10"/>
       <c r="O156" s="10"/>
     </row>
-    <row r="157" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A157" s="10"/>
       <c r="B157" s="10"/>
       <c r="C157" s="10"/>
@@ -4621,7 +4650,7 @@
       <c r="N157" s="10"/>
       <c r="O157" s="10"/>
     </row>
-    <row r="158" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A158" s="10"/>
       <c r="B158" s="10"/>
       <c r="C158" s="10"/>
@@ -4641,7 +4670,7 @@
       <c r="N158" s="10"/>
       <c r="O158" s="10"/>
     </row>
-    <row r="159" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A159" s="10"/>
       <c r="B159" s="10"/>
       <c r="C159" s="10"/>
@@ -4661,7 +4690,7 @@
       <c r="N159" s="10"/>
       <c r="O159" s="10"/>
     </row>
-    <row r="160" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A160" s="10"/>
       <c r="B160" s="10"/>
       <c r="C160" s="10"/>
@@ -4681,7 +4710,7 @@
       <c r="N160" s="10"/>
       <c r="O160" s="10"/>
     </row>
-    <row r="161" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A161" s="10"/>
       <c r="B161" s="10"/>
       <c r="C161" s="10"/>
@@ -4701,7 +4730,7 @@
       <c r="N161" s="10"/>
       <c r="O161" s="10"/>
     </row>
-    <row r="162" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A162" s="10"/>
       <c r="B162" s="10"/>
       <c r="C162" s="10"/>
@@ -4721,7 +4750,7 @@
       <c r="N162" s="10"/>
       <c r="O162" s="10"/>
     </row>
-    <row r="163" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A163" s="10"/>
       <c r="B163" s="10"/>
       <c r="C163" s="10"/>
@@ -4741,7 +4770,7 @@
       <c r="N163" s="10"/>
       <c r="O163" s="10"/>
     </row>
-    <row r="164" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A164" s="10"/>
       <c r="B164" s="10"/>
       <c r="C164" s="10"/>
@@ -4761,7 +4790,7 @@
       <c r="N164" s="10"/>
       <c r="O164" s="10"/>
     </row>
-    <row r="165" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A165" s="10"/>
       <c r="B165" s="10"/>
       <c r="C165" s="10"/>
@@ -4781,7 +4810,7 @@
       <c r="N165" s="10"/>
       <c r="O165" s="10"/>
     </row>
-    <row r="166" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A166" s="10"/>
       <c r="B166" s="10"/>
       <c r="C166" s="10"/>
@@ -4801,7 +4830,7 @@
       <c r="N166" s="10"/>
       <c r="O166" s="10"/>
     </row>
-    <row r="167" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A167" s="10"/>
       <c r="B167" s="10"/>
       <c r="C167" s="10"/>
@@ -4821,7 +4850,7 @@
       <c r="N167" s="10"/>
       <c r="O167" s="10"/>
     </row>
-    <row r="168" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A168" s="10"/>
       <c r="B168" s="10"/>
       <c r="C168" s="10"/>
@@ -4841,7 +4870,7 @@
       <c r="N168" s="10"/>
       <c r="O168" s="10"/>
     </row>
-    <row r="169" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A169" s="10"/>
       <c r="B169" s="10"/>
       <c r="C169" s="10"/>
@@ -4861,7 +4890,7 @@
       <c r="N169" s="10"/>
       <c r="O169" s="10"/>
     </row>
-    <row r="170" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A170" s="10"/>
       <c r="B170" s="10"/>
       <c r="C170" s="10"/>
@@ -4881,7 +4910,7 @@
       <c r="N170" s="10"/>
       <c r="O170" s="10"/>
     </row>
-    <row r="171" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A171" s="10"/>
       <c r="B171" s="10"/>
       <c r="C171" s="10"/>
@@ -4901,7 +4930,7 @@
       <c r="N171" s="10"/>
       <c r="O171" s="10"/>
     </row>
-    <row r="172" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A172" s="10"/>
       <c r="B172" s="10"/>
       <c r="C172" s="10"/>
@@ -4921,7 +4950,7 @@
       <c r="N172" s="10"/>
       <c r="O172" s="10"/>
     </row>
-    <row r="173" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A173" s="10"/>
       <c r="B173" s="10"/>
       <c r="C173" s="10"/>
@@ -4941,7 +4970,7 @@
       <c r="N173" s="10"/>
       <c r="O173" s="10"/>
     </row>
-    <row r="174" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A174" s="10"/>
       <c r="B174" s="10"/>
       <c r="C174" s="10"/>
@@ -4961,7 +4990,7 @@
       <c r="N174" s="10"/>
       <c r="O174" s="10"/>
     </row>
-    <row r="175" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A175" s="10"/>
       <c r="B175" s="10"/>
       <c r="C175" s="10"/>
@@ -4981,7 +5010,7 @@
       <c r="N175" s="10"/>
       <c r="O175" s="10"/>
     </row>
-    <row r="176" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A176" s="10"/>
       <c r="B176" s="10"/>
       <c r="C176" s="10"/>
@@ -5001,7 +5030,7 @@
       <c r="N176" s="10"/>
       <c r="O176" s="10"/>
     </row>
-    <row r="177" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A177" s="10"/>
       <c r="B177" s="10"/>
       <c r="C177" s="10"/>
@@ -5021,7 +5050,7 @@
       <c r="N177" s="10"/>
       <c r="O177" s="10"/>
     </row>
-    <row r="178" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A178" s="10"/>
       <c r="B178" s="10"/>
       <c r="C178" s="10"/>
@@ -5041,7 +5070,7 @@
       <c r="N178" s="10"/>
       <c r="O178" s="10"/>
     </row>
-    <row r="179" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A179" s="10"/>
       <c r="B179" s="10"/>
       <c r="C179" s="10"/>
@@ -5061,7 +5090,7 @@
       <c r="N179" s="10"/>
       <c r="O179" s="10"/>
     </row>
-    <row r="180" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A180" s="10"/>
       <c r="B180" s="10"/>
       <c r="C180" s="10"/>
@@ -5081,7 +5110,7 @@
       <c r="N180" s="10"/>
       <c r="O180" s="10"/>
     </row>
-    <row r="181" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A181" s="10"/>
       <c r="B181" s="10"/>
       <c r="C181" s="10"/>
@@ -5101,7 +5130,7 @@
       <c r="N181" s="10"/>
       <c r="O181" s="10"/>
     </row>
-    <row r="182" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A182" s="10"/>
       <c r="B182" s="10"/>
       <c r="C182" s="10"/>
@@ -5121,7 +5150,7 @@
       <c r="N182" s="10"/>
       <c r="O182" s="10"/>
     </row>
-    <row r="183" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A183" s="10"/>
       <c r="B183" s="10"/>
       <c r="C183" s="10"/>
@@ -5141,7 +5170,7 @@
       <c r="N183" s="10"/>
       <c r="O183" s="10"/>
     </row>
-    <row r="184" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A184" s="10"/>
       <c r="B184" s="10"/>
       <c r="C184" s="10"/>
@@ -5161,7 +5190,7 @@
       <c r="N184" s="10"/>
       <c r="O184" s="10"/>
     </row>
-    <row r="185" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A185" s="10"/>
       <c r="B185" s="10"/>
       <c r="C185" s="10"/>
@@ -5181,7 +5210,7 @@
       <c r="N185" s="10"/>
       <c r="O185" s="10"/>
     </row>
-    <row r="186" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A186" s="10"/>
       <c r="B186" s="10"/>
       <c r="C186" s="10"/>
@@ -5201,7 +5230,7 @@
       <c r="N186" s="10"/>
       <c r="O186" s="10"/>
     </row>
-    <row r="187" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A187" s="10"/>
       <c r="B187" s="10"/>
       <c r="C187" s="10"/>
@@ -5221,7 +5250,7 @@
       <c r="N187" s="10"/>
       <c r="O187" s="10"/>
     </row>
-    <row r="188" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A188" s="10"/>
       <c r="B188" s="10"/>
       <c r="C188" s="10"/>
@@ -5241,7 +5270,7 @@
       <c r="N188" s="10"/>
       <c r="O188" s="10"/>
     </row>
-    <row r="189" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A189" s="10"/>
       <c r="B189" s="10"/>
       <c r="C189" s="10"/>
@@ -5261,7 +5290,7 @@
       <c r="N189" s="10"/>
       <c r="O189" s="10"/>
     </row>
-    <row r="190" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A190" s="10"/>
       <c r="B190" s="10"/>
       <c r="C190" s="10"/>
@@ -5281,7 +5310,7 @@
       <c r="N190" s="10"/>
       <c r="O190" s="10"/>
     </row>
-    <row r="191" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A191" s="10"/>
       <c r="B191" s="10"/>
       <c r="C191" s="10"/>
@@ -5301,7 +5330,7 @@
       <c r="N191" s="10"/>
       <c r="O191" s="10"/>
     </row>
-    <row r="192" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A192" s="10"/>
       <c r="B192" s="10"/>
       <c r="C192" s="10"/>
@@ -5321,7 +5350,7 @@
       <c r="N192" s="10"/>
       <c r="O192" s="10"/>
     </row>
-    <row r="193" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A193" s="10"/>
       <c r="B193" s="10"/>
       <c r="C193" s="10"/>
@@ -5341,7 +5370,7 @@
       <c r="N193" s="10"/>
       <c r="O193" s="10"/>
     </row>
-    <row r="194" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A194" s="10"/>
       <c r="B194" s="10"/>
       <c r="C194" s="10"/>
@@ -5361,7 +5390,7 @@
       <c r="N194" s="10"/>
       <c r="O194" s="10"/>
     </row>
-    <row r="195" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A195" s="10"/>
       <c r="B195" s="10"/>
       <c r="C195" s="10"/>
@@ -5381,7 +5410,7 @@
       <c r="N195" s="10"/>
       <c r="O195" s="10"/>
     </row>
-    <row r="196" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A196" s="10"/>
       <c r="B196" s="10"/>
       <c r="C196" s="10"/>
@@ -5401,7 +5430,7 @@
       <c r="N196" s="10"/>
       <c r="O196" s="10"/>
     </row>
-    <row r="197" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A197" s="10"/>
       <c r="B197" s="10"/>
       <c r="C197" s="10"/>
@@ -5421,7 +5450,7 @@
       <c r="N197" s="10"/>
       <c r="O197" s="10"/>
     </row>
-    <row r="198" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A198" s="10"/>
       <c r="B198" s="10"/>
       <c r="C198" s="10"/>
@@ -5441,7 +5470,7 @@
       <c r="N198" s="10"/>
       <c r="O198" s="10"/>
     </row>
-    <row r="199" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A199" s="10"/>
       <c r="B199" s="10"/>
       <c r="C199" s="10"/>
@@ -5461,7 +5490,7 @@
       <c r="N199" s="10"/>
       <c r="O199" s="10"/>
     </row>
-    <row r="200" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A200" s="10"/>
       <c r="B200" s="10"/>
       <c r="C200" s="10"/>
@@ -5481,7 +5510,7 @@
       <c r="N200" s="10"/>
       <c r="O200" s="10"/>
     </row>
-    <row r="201" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A201" s="10"/>
       <c r="B201" s="10"/>
       <c r="C201" s="10"/>
@@ -5501,7 +5530,7 @@
       <c r="N201" s="10"/>
       <c r="O201" s="10"/>
     </row>
-    <row r="202" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A202" s="10"/>
       <c r="B202" s="10"/>
       <c r="C202" s="10"/>
@@ -5521,7 +5550,7 @@
       <c r="N202" s="10"/>
       <c r="O202" s="10"/>
     </row>
-    <row r="203" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A203" s="10"/>
       <c r="B203" s="10"/>
       <c r="C203" s="10"/>
@@ -5541,7 +5570,7 @@
       <c r="N203" s="10"/>
       <c r="O203" s="10"/>
     </row>
-    <row r="204" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A204" s="10"/>
       <c r="B204" s="10"/>
       <c r="C204" s="10"/>
@@ -5561,7 +5590,7 @@
       <c r="N204" s="10"/>
       <c r="O204" s="10"/>
     </row>
-    <row r="205" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A205" s="10"/>
       <c r="B205" s="10"/>
       <c r="C205" s="10"/>
@@ -5581,7 +5610,7 @@
       <c r="N205" s="10"/>
       <c r="O205" s="10"/>
     </row>
-    <row r="206" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A206" s="10"/>
       <c r="B206" s="10"/>
       <c r="C206" s="10"/>
@@ -5601,7 +5630,7 @@
       <c r="N206" s="10"/>
       <c r="O206" s="10"/>
     </row>
-    <row r="207" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A207" s="10"/>
       <c r="B207" s="10"/>
       <c r="C207" s="10"/>
@@ -5621,7 +5650,7 @@
       <c r="N207" s="10"/>
       <c r="O207" s="10"/>
     </row>
-    <row r="208" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A208" s="10"/>
       <c r="B208" s="10"/>
       <c r="C208" s="10"/>
@@ -5641,7 +5670,7 @@
       <c r="N208" s="10"/>
       <c r="O208" s="10"/>
     </row>
-    <row r="209" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A209" s="10"/>
       <c r="B209" s="10"/>
       <c r="C209" s="10"/>
@@ -5661,7 +5690,7 @@
       <c r="N209" s="10"/>
       <c r="O209" s="10"/>
     </row>
-    <row r="210" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A210" s="10"/>
       <c r="B210" s="10"/>
       <c r="C210" s="10"/>
@@ -5681,7 +5710,7 @@
       <c r="N210" s="10"/>
       <c r="O210" s="10"/>
     </row>
-    <row r="211" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A211" s="10"/>
       <c r="B211" s="10"/>
       <c r="C211" s="10"/>
@@ -5701,7 +5730,7 @@
       <c r="N211" s="10"/>
       <c r="O211" s="10"/>
     </row>
-    <row r="212" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A212" s="10"/>
       <c r="B212" s="10"/>
       <c r="C212" s="10"/>
@@ -5721,7 +5750,7 @@
       <c r="N212" s="10"/>
       <c r="O212" s="10"/>
     </row>
-    <row r="213" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A213" s="10"/>
       <c r="B213" s="10"/>
       <c r="C213" s="10"/>
@@ -5741,7 +5770,7 @@
       <c r="N213" s="10"/>
       <c r="O213" s="10"/>
     </row>
-    <row r="214" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A214" s="10"/>
       <c r="B214" s="10"/>
       <c r="C214" s="10"/>
@@ -5761,7 +5790,7 @@
       <c r="N214" s="10"/>
       <c r="O214" s="10"/>
     </row>
-    <row r="215" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A215" s="10"/>
       <c r="B215" s="10"/>
       <c r="C215" s="10"/>
@@ -5781,7 +5810,7 @@
       <c r="N215" s="10"/>
       <c r="O215" s="10"/>
     </row>
-    <row r="216" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A216" s="10"/>
       <c r="B216" s="10"/>
       <c r="C216" s="10"/>
@@ -5801,7 +5830,7 @@
       <c r="N216" s="10"/>
       <c r="O216" s="10"/>
     </row>
-    <row r="217" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A217" s="10"/>
       <c r="B217" s="10"/>
       <c r="C217" s="10"/>
@@ -5821,7 +5850,7 @@
       <c r="N217" s="10"/>
       <c r="O217" s="10"/>
     </row>
-    <row r="218" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A218" s="10"/>
       <c r="B218" s="10"/>
       <c r="C218" s="10"/>
@@ -5841,7 +5870,7 @@
       <c r="N218" s="10"/>
       <c r="O218" s="10"/>
     </row>
-    <row r="219" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A219" s="10"/>
       <c r="B219" s="10"/>
       <c r="C219" s="10"/>
@@ -5861,7 +5890,7 @@
       <c r="N219" s="10"/>
       <c r="O219" s="10"/>
     </row>
-    <row r="220" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A220" s="10"/>
       <c r="B220" s="10"/>
       <c r="C220" s="10"/>
@@ -5881,7 +5910,7 @@
       <c r="N220" s="10"/>
       <c r="O220" s="10"/>
     </row>
-    <row r="221" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A221" s="10"/>
       <c r="B221" s="10"/>
       <c r="C221" s="10"/>
@@ -5901,7 +5930,7 @@
       <c r="N221" s="10"/>
       <c r="O221" s="10"/>
     </row>
-    <row r="222" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A222" s="10"/>
       <c r="B222" s="10"/>
       <c r="C222" s="10"/>
@@ -5921,7 +5950,7 @@
       <c r="N222" s="10"/>
       <c r="O222" s="10"/>
     </row>
-    <row r="223" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A223" s="10"/>
       <c r="B223" s="10"/>
       <c r="C223" s="10"/>
@@ -5941,7 +5970,7 @@
       <c r="N223" s="10"/>
       <c r="O223" s="10"/>
     </row>
-    <row r="224" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A224" s="10"/>
       <c r="B224" s="10"/>
       <c r="C224" s="10"/>
@@ -5961,7 +5990,7 @@
       <c r="N224" s="10"/>
       <c r="O224" s="10"/>
     </row>
-    <row r="225" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A225" s="10"/>
       <c r="B225" s="10"/>
       <c r="C225" s="10"/>
@@ -5981,7 +6010,7 @@
       <c r="N225" s="10"/>
       <c r="O225" s="10"/>
     </row>
-    <row r="226" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A226" s="10"/>
       <c r="B226" s="10"/>
       <c r="C226" s="10"/>
@@ -6001,7 +6030,7 @@
       <c r="N226" s="10"/>
       <c r="O226" s="10"/>
     </row>
-    <row r="227" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A227" s="10"/>
       <c r="B227" s="10"/>
       <c r="C227" s="10"/>
@@ -6021,7 +6050,7 @@
       <c r="N227" s="10"/>
       <c r="O227" s="10"/>
     </row>
-    <row r="228" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A228" s="10"/>
       <c r="B228" s="10"/>
       <c r="C228" s="10"/>
@@ -6041,7 +6070,7 @@
       <c r="N228" s="10"/>
       <c r="O228" s="10"/>
     </row>
-    <row r="229" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A229" s="10"/>
       <c r="B229" s="10"/>
       <c r="C229" s="10"/>
@@ -6061,7 +6090,7 @@
       <c r="N229" s="10"/>
       <c r="O229" s="10"/>
     </row>
-    <row r="230" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A230" s="10"/>
       <c r="B230" s="10"/>
       <c r="C230" s="10"/>
@@ -6081,7 +6110,7 @@
       <c r="N230" s="10"/>
       <c r="O230" s="10"/>
     </row>
-    <row r="231" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A231" s="10"/>
       <c r="B231" s="10"/>
       <c r="C231" s="10"/>
@@ -6101,7 +6130,7 @@
       <c r="N231" s="10"/>
       <c r="O231" s="10"/>
     </row>
-    <row r="232" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A232" s="10"/>
       <c r="B232" s="10"/>
       <c r="C232" s="10"/>
@@ -6121,7 +6150,7 @@
       <c r="N232" s="10"/>
       <c r="O232" s="10"/>
     </row>
-    <row r="233" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A233" s="10"/>
       <c r="B233" s="10"/>
       <c r="C233" s="10"/>
@@ -6141,7 +6170,7 @@
       <c r="N233" s="10"/>
       <c r="O233" s="10"/>
     </row>
-    <row r="234" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A234" s="10"/>
       <c r="B234" s="10"/>
       <c r="C234" s="10"/>
@@ -6161,7 +6190,7 @@
       <c r="N234" s="10"/>
       <c r="O234" s="10"/>
     </row>
-    <row r="235" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A235" s="10"/>
       <c r="B235" s="10"/>
       <c r="C235" s="10"/>
@@ -6181,7 +6210,7 @@
       <c r="N235" s="10"/>
       <c r="O235" s="10"/>
     </row>
-    <row r="236" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A236" s="10"/>
       <c r="B236" s="10"/>
       <c r="C236" s="10"/>
@@ -6201,7 +6230,7 @@
       <c r="N236" s="10"/>
       <c r="O236" s="10"/>
     </row>
-    <row r="237" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A237" s="10"/>
       <c r="B237" s="10"/>
       <c r="C237" s="10"/>
@@ -6221,7 +6250,7 @@
       <c r="N237" s="10"/>
       <c r="O237" s="10"/>
     </row>
-    <row r="238" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A238" s="10"/>
       <c r="B238" s="10"/>
       <c r="C238" s="10"/>
@@ -6241,7 +6270,7 @@
       <c r="N238" s="10"/>
       <c r="O238" s="10"/>
     </row>
-    <row r="239" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A239" s="10"/>
       <c r="B239" s="10"/>
       <c r="C239" s="10"/>
@@ -6261,7 +6290,7 @@
       <c r="N239" s="10"/>
       <c r="O239" s="10"/>
     </row>
-    <row r="240" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A240" s="10"/>
       <c r="B240" s="10"/>
       <c r="C240" s="10"/>
@@ -6281,7 +6310,7 @@
       <c r="N240" s="10"/>
       <c r="O240" s="10"/>
     </row>
-    <row r="241" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A241" s="10"/>
       <c r="B241" s="10"/>
       <c r="C241" s="10"/>
@@ -6301,7 +6330,7 @@
       <c r="N241" s="10"/>
       <c r="O241" s="10"/>
     </row>
-    <row r="242" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A242" s="10"/>
       <c r="B242" s="10"/>
       <c r="C242" s="10"/>
@@ -6321,7 +6350,7 @@
       <c r="N242" s="10"/>
       <c r="O242" s="10"/>
     </row>
-    <row r="243" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A243" s="10"/>
       <c r="B243" s="10"/>
       <c r="C243" s="10"/>
@@ -6341,7 +6370,7 @@
       <c r="N243" s="10"/>
       <c r="O243" s="10"/>
     </row>
-    <row r="244" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A244" s="10"/>
       <c r="B244" s="10"/>
       <c r="C244" s="10"/>
@@ -6361,7 +6390,7 @@
       <c r="N244" s="10"/>
       <c r="O244" s="10"/>
     </row>
-    <row r="245" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A245" s="10"/>
       <c r="B245" s="10"/>
       <c r="C245" s="10"/>
@@ -6381,7 +6410,7 @@
       <c r="N245" s="10"/>
       <c r="O245" s="10"/>
     </row>
-    <row r="246" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A246" s="10"/>
       <c r="B246" s="10"/>
       <c r="C246" s="10"/>
@@ -6401,7 +6430,7 @@
       <c r="N246" s="10"/>
       <c r="O246" s="10"/>
     </row>
-    <row r="247" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A247" s="10"/>
       <c r="B247" s="10"/>
       <c r="C247" s="10"/>
@@ -6421,7 +6450,7 @@
       <c r="N247" s="10"/>
       <c r="O247" s="10"/>
     </row>
-    <row r="248" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A248" s="10"/>
       <c r="B248" s="10"/>
       <c r="C248" s="10"/>
@@ -6441,7 +6470,7 @@
       <c r="N248" s="10"/>
       <c r="O248" s="10"/>
     </row>
-    <row r="249" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A249" s="10"/>
       <c r="B249" s="10"/>
       <c r="C249" s="10"/>
@@ -6461,7 +6490,7 @@
       <c r="N249" s="10"/>
       <c r="O249" s="10"/>
     </row>
-    <row r="250" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A250" s="10"/>
       <c r="B250" s="10"/>
       <c r="C250" s="10"/>
@@ -6481,7 +6510,7 @@
       <c r="N250" s="10"/>
       <c r="O250" s="10"/>
     </row>
-    <row r="251" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A251" s="10"/>
       <c r="B251" s="10"/>
       <c r="C251" s="10"/>
@@ -6501,7 +6530,7 @@
       <c r="N251" s="10"/>
       <c r="O251" s="10"/>
     </row>
-    <row r="252" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A252" s="10"/>
       <c r="B252" s="10"/>
       <c r="C252" s="10"/>
@@ -6521,7 +6550,7 @@
       <c r="N252" s="10"/>
       <c r="O252" s="10"/>
     </row>
-    <row r="253" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A253" s="10"/>
       <c r="B253" s="10"/>
       <c r="C253" s="10"/>
@@ -6541,7 +6570,7 @@
       <c r="N253" s="10"/>
       <c r="O253" s="10"/>
     </row>
-    <row r="254" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A254" s="10"/>
       <c r="B254" s="10"/>
       <c r="C254" s="10"/>
@@ -6561,7 +6590,7 @@
       <c r="N254" s="10"/>
       <c r="O254" s="10"/>
     </row>
-    <row r="255" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A255" s="10"/>
       <c r="B255" s="10"/>
       <c r="C255" s="10"/>
@@ -6581,7 +6610,7 @@
       <c r="N255" s="10"/>
       <c r="O255" s="10"/>
     </row>
-    <row r="256" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A256" s="10"/>
       <c r="B256" s="10"/>
       <c r="C256" s="10"/>
@@ -6601,7 +6630,7 @@
       <c r="N256" s="10"/>
       <c r="O256" s="10"/>
     </row>
-    <row r="257" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A257" s="10"/>
       <c r="B257" s="10"/>
       <c r="C257" s="10"/>
@@ -6621,7 +6650,7 @@
       <c r="N257" s="10"/>
       <c r="O257" s="10"/>
     </row>
-    <row r="258" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A258" s="10"/>
       <c r="B258" s="10"/>
       <c r="C258" s="10"/>
@@ -6641,7 +6670,7 @@
       <c r="N258" s="10"/>
       <c r="O258" s="10"/>
     </row>
-    <row r="259" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A259" s="10"/>
       <c r="B259" s="10"/>
       <c r="C259" s="10"/>
@@ -6661,7 +6690,7 @@
       <c r="N259" s="10"/>
       <c r="O259" s="10"/>
     </row>
-    <row r="260" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A260" s="10"/>
       <c r="B260" s="10"/>
       <c r="C260" s="10"/>
@@ -6681,7 +6710,7 @@
       <c r="N260" s="10"/>
       <c r="O260" s="10"/>
     </row>
-    <row r="261" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A261" s="10"/>
       <c r="B261" s="10"/>
       <c r="C261" s="10"/>
@@ -6701,7 +6730,7 @@
       <c r="N261" s="10"/>
       <c r="O261" s="10"/>
     </row>
-    <row r="262" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A262" s="10"/>
       <c r="B262" s="10"/>
       <c r="C262" s="10"/>
@@ -6721,7 +6750,7 @@
       <c r="N262" s="10"/>
       <c r="O262" s="10"/>
     </row>
-    <row r="263" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A263" s="10"/>
       <c r="B263" s="10"/>
       <c r="C263" s="10"/>
@@ -6741,7 +6770,7 @@
       <c r="N263" s="10"/>
       <c r="O263" s="10"/>
     </row>
-    <row r="264" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A264" s="10"/>
       <c r="B264" s="10"/>
       <c r="C264" s="10"/>
@@ -6761,7 +6790,7 @@
       <c r="N264" s="10"/>
       <c r="O264" s="10"/>
     </row>
-    <row r="265" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A265" s="10"/>
       <c r="B265" s="10"/>
       <c r="C265" s="10"/>
@@ -6781,7 +6810,7 @@
       <c r="N265" s="10"/>
       <c r="O265" s="10"/>
     </row>
-    <row r="266" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A266" s="10"/>
       <c r="B266" s="10"/>
       <c r="C266" s="10"/>
@@ -6801,7 +6830,7 @@
       <c r="N266" s="10"/>
       <c r="O266" s="10"/>
     </row>
-    <row r="267" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A267" s="10"/>
       <c r="B267" s="10"/>
       <c r="C267" s="10"/>
@@ -6821,7 +6850,7 @@
       <c r="N267" s="10"/>
       <c r="O267" s="10"/>
     </row>
-    <row r="268" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A268" s="10"/>
       <c r="B268" s="10"/>
       <c r="C268" s="10"/>
@@ -6841,7 +6870,7 @@
       <c r="N268" s="10"/>
       <c r="O268" s="10"/>
     </row>
-    <row r="269" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A269" s="10"/>
       <c r="B269" s="10"/>
       <c r="C269" s="10"/>
@@ -6861,7 +6890,7 @@
       <c r="N269" s="10"/>
       <c r="O269" s="10"/>
     </row>
-    <row r="270" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A270" s="10"/>
       <c r="B270" s="10"/>
       <c r="C270" s="10"/>
@@ -6881,7 +6910,7 @@
       <c r="N270" s="10"/>
       <c r="O270" s="10"/>
     </row>
-    <row r="271" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A271" s="10"/>
       <c r="B271" s="10"/>
       <c r="C271" s="10"/>
@@ -6901,7 +6930,7 @@
       <c r="N271" s="10"/>
       <c r="O271" s="10"/>
     </row>
-    <row r="272" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A272" s="10"/>
       <c r="B272" s="10"/>
       <c r="C272" s="10"/>
@@ -6921,7 +6950,7 @@
       <c r="N272" s="10"/>
       <c r="O272" s="10"/>
     </row>
-    <row r="273" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A273" s="10"/>
       <c r="B273" s="10"/>
       <c r="C273" s="10"/>
@@ -6941,7 +6970,7 @@
       <c r="N273" s="10"/>
       <c r="O273" s="10"/>
     </row>
-    <row r="274" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A274" s="10"/>
       <c r="B274" s="10"/>
       <c r="C274" s="10"/>
@@ -6961,7 +6990,7 @@
       <c r="N274" s="10"/>
       <c r="O274" s="10"/>
     </row>
-    <row r="275" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A275" s="10"/>
       <c r="B275" s="10"/>
       <c r="C275" s="10"/>
@@ -6981,7 +7010,7 @@
       <c r="N275" s="10"/>
       <c r="O275" s="10"/>
     </row>
-    <row r="276" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A276" s="10"/>
       <c r="B276" s="10"/>
       <c r="C276" s="10"/>
@@ -7001,7 +7030,7 @@
       <c r="N276" s="10"/>
       <c r="O276" s="10"/>
     </row>
-    <row r="277" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A277" s="10"/>
       <c r="B277" s="10"/>
       <c r="C277" s="10"/>
@@ -7021,7 +7050,7 @@
       <c r="N277" s="10"/>
       <c r="O277" s="10"/>
     </row>
-    <row r="278" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A278" s="10"/>
       <c r="B278" s="10"/>
       <c r="C278" s="10"/>
@@ -7041,7 +7070,7 @@
       <c r="N278" s="10"/>
       <c r="O278" s="10"/>
     </row>
-    <row r="279" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A279" s="10"/>
       <c r="B279" s="10"/>
       <c r="C279" s="10"/>
@@ -7061,7 +7090,7 @@
       <c r="N279" s="10"/>
       <c r="O279" s="10"/>
     </row>
-    <row r="280" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A280" s="10"/>
       <c r="B280" s="10"/>
       <c r="C280" s="10"/>
@@ -7081,7 +7110,7 @@
       <c r="N280" s="10"/>
       <c r="O280" s="10"/>
     </row>
-    <row r="281" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A281" s="10"/>
       <c r="B281" s="10"/>
       <c r="C281" s="10"/>
@@ -7101,7 +7130,7 @@
       <c r="N281" s="10"/>
       <c r="O281" s="10"/>
     </row>
-    <row r="282" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A282" s="10"/>
       <c r="B282" s="10"/>
       <c r="C282" s="10"/>
@@ -7121,7 +7150,7 @@
       <c r="N282" s="10"/>
       <c r="O282" s="10"/>
     </row>
-    <row r="283" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A283" s="10"/>
       <c r="B283" s="10"/>
       <c r="C283" s="10"/>
@@ -7141,7 +7170,7 @@
       <c r="N283" s="10"/>
       <c r="O283" s="10"/>
     </row>
-    <row r="284" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A284" s="10"/>
       <c r="B284" s="10"/>
       <c r="C284" s="10"/>
@@ -7161,7 +7190,7 @@
       <c r="N284" s="10"/>
       <c r="O284" s="10"/>
     </row>
-    <row r="285" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A285" s="10"/>
       <c r="B285" s="10"/>
       <c r="C285" s="10"/>
@@ -7181,7 +7210,7 @@
       <c r="N285" s="10"/>
       <c r="O285" s="10"/>
     </row>
-    <row r="286" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A286" s="10"/>
       <c r="B286" s="10"/>
       <c r="C286" s="10"/>
@@ -7201,7 +7230,7 @@
       <c r="N286" s="10"/>
       <c r="O286" s="10"/>
     </row>
-    <row r="287" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A287" s="10"/>
       <c r="B287" s="10"/>
       <c r="C287" s="10"/>
@@ -7221,7 +7250,7 @@
       <c r="N287" s="10"/>
       <c r="O287" s="10"/>
     </row>
-    <row r="288" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A288" s="10"/>
       <c r="B288" s="10"/>
       <c r="C288" s="10"/>
@@ -7241,7 +7270,7 @@
       <c r="N288" s="10"/>
       <c r="O288" s="10"/>
     </row>
-    <row r="289" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A289" s="10"/>
       <c r="B289" s="10"/>
       <c r="C289" s="10"/>
@@ -7261,7 +7290,7 @@
       <c r="N289" s="10"/>
       <c r="O289" s="10"/>
     </row>
-    <row r="290" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A290" s="10"/>
       <c r="B290" s="10"/>
       <c r="C290" s="10"/>
@@ -7281,7 +7310,7 @@
       <c r="N290" s="10"/>
       <c r="O290" s="10"/>
     </row>
-    <row r="291" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A291" s="10"/>
       <c r="B291" s="10"/>
       <c r="C291" s="10"/>
@@ -7301,7 +7330,7 @@
       <c r="N291" s="10"/>
       <c r="O291" s="10"/>
     </row>
-    <row r="292" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A292" s="10"/>
       <c r="B292" s="10"/>
       <c r="C292" s="10"/>
@@ -7321,7 +7350,7 @@
       <c r="N292" s="10"/>
       <c r="O292" s="10"/>
     </row>
-    <row r="293" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A293" s="10"/>
       <c r="B293" s="10"/>
       <c r="C293" s="10"/>
@@ -7341,7 +7370,7 @@
       <c r="N293" s="10"/>
       <c r="O293" s="10"/>
     </row>
-    <row r="294" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A294" s="10"/>
       <c r="B294" s="10"/>
       <c r="C294" s="10"/>
@@ -7361,7 +7390,7 @@
       <c r="N294" s="10"/>
       <c r="O294" s="10"/>
     </row>
-    <row r="295" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A295" s="10"/>
       <c r="B295" s="10"/>
       <c r="C295" s="10"/>
@@ -7381,7 +7410,7 @@
       <c r="N295" s="10"/>
       <c r="O295" s="10"/>
     </row>
-    <row r="296" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A296" s="10"/>
       <c r="B296" s="10"/>
       <c r="C296" s="10"/>
@@ -7401,7 +7430,7 @@
       <c r="N296" s="10"/>
       <c r="O296" s="10"/>
     </row>
-    <row r="297" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A297" s="10"/>
       <c r="B297" s="10"/>
       <c r="C297" s="10"/>
@@ -7421,7 +7450,7 @@
       <c r="N297" s="10"/>
       <c r="O297" s="10"/>
     </row>
-    <row r="298" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A298" s="10"/>
       <c r="B298" s="10"/>
       <c r="C298" s="10"/>
@@ -7441,7 +7470,7 @@
       <c r="N298" s="10"/>
       <c r="O298" s="10"/>
     </row>
-    <row r="299" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A299" s="10"/>
       <c r="B299" s="10"/>
       <c r="C299" s="10"/>
@@ -7461,7 +7490,7 @@
       <c r="N299" s="10"/>
       <c r="O299" s="10"/>
     </row>
-    <row r="300" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A300" s="10"/>
       <c r="B300" s="10"/>
       <c r="C300" s="10"/>
@@ -7481,7 +7510,7 @@
       <c r="N300" s="10"/>
       <c r="O300" s="10"/>
     </row>
-    <row r="301" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A301" s="10"/>
       <c r="B301" s="10"/>
       <c r="C301" s="10"/>
@@ -7501,7 +7530,7 @@
       <c r="N301" s="10"/>
       <c r="O301" s="10"/>
     </row>
-    <row r="302" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A302" s="10"/>
       <c r="B302" s="10"/>
       <c r="C302" s="10"/>
@@ -7521,7 +7550,7 @@
       <c r="N302" s="10"/>
       <c r="O302" s="10"/>
     </row>
-    <row r="303" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A303" s="10"/>
       <c r="B303" s="10"/>
       <c r="C303" s="10"/>
@@ -7541,7 +7570,7 @@
       <c r="N303" s="10"/>
       <c r="O303" s="10"/>
     </row>
-    <row r="304" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A304" s="10"/>
       <c r="B304" s="10"/>
       <c r="C304" s="10"/>
@@ -7598,7 +7627,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -7606,7 +7635,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -7614,139 +7643,139 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D4" s="9"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="12">
         <v>10</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D5" s="12"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" s="12">
         <v>10</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D6" s="12"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="12">
         <v>10</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D7" s="12"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="12">
         <v>20</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D8" s="12"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B9" s="12">
         <v>10</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D9" s="12"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B10" s="12">
         <v>10</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D10" s="12"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B11" s="12">
         <v>10</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D11" s="12"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B12" s="12">
         <v>5</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D12" s="12"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B13" s="12">
         <v>5</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D13" s="12"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B14" s="12">
         <v>10</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D14" s="12"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B15" s="13">
         <f>SUM(B5:B14)</f>
@@ -7755,7 +7784,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -7789,7 +7818,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7803,7 +7832,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7817,34 +7846,34 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>11</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -13296,7 +13325,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -13305,7 +13334,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -13314,7 +13343,7 @@
     </row>
     <row r="3" ht="28.05" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B3"/>
       <c r="C3"/>
@@ -13323,41 +13352,41 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="7:11" x14ac:dyDescent="0.25">
       <c r="G4" s="17" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H4"/>
       <c r="J4" s="17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K4"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -13367,13 +13396,13 @@
       <c r="D6" s="22"/>
       <c r="E6" s="20"/>
       <c r="G6" s="23" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="K6" s="26">
         <f>SUMIF($A$6:$A$305,"panel",$C$6:$C$305)</f>
@@ -13387,13 +13416,13 @@
       <c r="D7" s="22"/>
       <c r="E7" s="20"/>
       <c r="G7" s="27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J7" s="29" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K7" s="30">
         <f>SUMIF($A$6:$A$305,"inverter",$C$6:$C$305)</f>
@@ -13407,13 +13436,13 @@
       <c r="D8" s="22"/>
       <c r="E8" s="20"/>
       <c r="G8" s="23" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="J8" s="25" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K8" s="26">
         <f>SUMIF($A$6:$A$305,"mekanik",$C$6:$C$305)</f>
@@ -13427,13 +13456,13 @@
       <c r="D9" s="22"/>
       <c r="E9" s="20"/>
       <c r="G9" s="27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K9" s="30">
         <f>SUMIF($A$6:$A$305,"elektrik_dc",$C$6:$C$305)</f>
@@ -13447,13 +13476,13 @@
       <c r="D10" s="22"/>
       <c r="E10" s="20"/>
       <c r="G10" s="23" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J10" s="25" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K10" s="26">
         <f>SUMIF($A$6:$A$305,"elektrik_ac",$C$6:$C$305)</f>
@@ -13467,13 +13496,13 @@
       <c r="D11" s="22"/>
       <c r="E11" s="20"/>
       <c r="G11" s="27" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H11" s="28" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="J11" s="29" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K11" s="30">
         <f>SUMIF($A$6:$A$305,"elektrik_og",$C$6:$C$305)</f>
@@ -13487,13 +13516,13 @@
       <c r="D12" s="22"/>
       <c r="E12" s="20"/>
       <c r="G12" s="23" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H12" s="24" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J12" s="25" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K12" s="26">
         <f>SUMIF($A$6:$A$305,"enh",$C$6:$C$305)</f>
@@ -13507,13 +13536,13 @@
       <c r="D13" s="22"/>
       <c r="E13" s="20"/>
       <c r="G13" s="27" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H13" s="28" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J13" s="29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K13" s="30">
         <f>SUMIF($A$6:$A$305,"altyapi",$C$6:$C$305)</f>
@@ -13527,13 +13556,13 @@
       <c r="D14" s="22"/>
       <c r="E14" s="20"/>
       <c r="G14" s="23" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H14" s="24" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="J14" s="25" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K14" s="26">
         <f>SUMIF($A$6:$A$305,"iscilik",$C$6:$C$305)</f>
@@ -13547,13 +13576,13 @@
       <c r="D15" s="22"/>
       <c r="E15" s="20"/>
       <c r="G15" s="27" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H15" s="28" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J15" s="29" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K15" s="30">
         <f>SUMIF($A$6:$A$305,"izin",$C$6:$C$305)</f>
@@ -13567,13 +13596,13 @@
       <c r="D16" s="22"/>
       <c r="E16" s="20"/>
       <c r="G16" s="23" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H16" s="24" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J16" s="25" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K16" s="26">
         <f>SUMIF($A$6:$A$305,"denetim",$C$6:$C$305)</f>
@@ -13587,13 +13616,13 @@
       <c r="D17" s="22"/>
       <c r="E17" s="20"/>
       <c r="G17" s="27" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H17" s="28" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="J17" s="29" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K17" s="30">
         <f>SUMIF($A$6:$A$305,"diger",$C$6:$C$305)</f>
@@ -13607,7 +13636,7 @@
       <c r="D18" s="22"/>
       <c r="E18" s="20"/>
       <c r="J18" s="31" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K18" s="32">
         <f>SUM(K6:K17)</f>
@@ -13628,7 +13657,7 @@
       <c r="D20" s="22"/>
       <c r="E20" s="20"/>
       <c r="J20" s="33" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="K20" s="34">
         <f>COUNTIF($A$6:$A$305,"&lt;&gt;")</f>
@@ -15677,7 +15706,7 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -15692,7 +15721,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -15707,37 +15736,37 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -19666,7 +19695,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.45" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -19676,120 +19705,122 @@
   <sheetData>
     <row r="1" ht="28.05" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
       <c r="D1"/>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
       <c r="D2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>132</v>
+        <v>134</v>
+      </c>
+      <c r="E5" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="6" ht="57" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="7" ht="28.5" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" ht="28.5" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>138</v>
+        <v>141</v>
+      </c>
+      <c r="E7" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="11" spans="3:3" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="3:3" x14ac:dyDescent="0.25"/>
+        <v>151</v>
+      </c>
+    </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C13" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C14" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C15" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>